<commit_message>
Update behavior and fix routes
</commit_message>
<xml_diff>
--- a/TrailsTimeline.xlsx
+++ b/TrailsTimeline.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vjsal\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6da5a9201bc5826c/Documentos/trails_orbal_atlas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54315043-5A41-45C0-BA2E-F1BBE0C76030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{54315043-5A41-45C0-BA2E-F1BBE0C76030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{25870A69-3C63-4034-AC28-CAF6CC882F34}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{B6393BEF-99C0-4DAE-AD63-40B518CD1F0D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{B6393BEF-99C0-4DAE-AD63-40B518CD1F0D}"/>
   </bookViews>
   <sheets>
     <sheet name="characters" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="117">
   <si>
     <t>char_id</t>
   </si>
@@ -378,9 +378,6 @@
     <t>Returning Home</t>
   </si>
   <si>
-    <t>Learned the airliner Linda has disappeared over Bose, which Cassius was aboard</t>
-  </si>
-  <si>
     <t>Get sent to Rolent to pickup a newspaper for Cassius</t>
   </si>
   <si>
@@ -391,6 +388,12 @@
   </si>
   <si>
     <t>Guiding Estelle and Josua on their missions</t>
+  </si>
+  <si>
+    <t>Learned the airliner Linde has disappeared over Bose, which Cassius was aboard</t>
+  </si>
+  <si>
+    <t>show_name</t>
   </si>
 </sst>
 </file>
@@ -449,6 +452,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -907,14 +914,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBE7F938-F724-45B1-B18D-82E13C0D228D}">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>16</v>
       </c>
@@ -933,8 +940,11 @@
       <c r="F1" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -948,7 +958,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>79</v>
       </c>
@@ -968,7 +978,7 @@
         <v>68.900000000000006</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>23</v>
       </c>
@@ -979,7 +989,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>39</v>
       </c>
@@ -999,7 +1009,7 @@
         <v>67.7</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>37</v>
       </c>
@@ -1018,8 +1028,11 @@
       <c r="F6">
         <v>69.2</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>41</v>
       </c>
@@ -1038,8 +1051,11 @@
       <c r="F7">
         <v>69.900000000000006</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>42</v>
       </c>
@@ -1059,7 +1075,7 @@
         <v>65.8</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>47</v>
       </c>
@@ -1078,8 +1094,11 @@
       <c r="F9">
         <v>70.599999999999994</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>55</v>
       </c>
@@ -1093,7 +1112,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>81</v>
       </c>
@@ -1159,7 +1178,7 @@
         <v>35</v>
       </c>
       <c r="D2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E2" t="s">
         <v>41</v>
@@ -1719,7 +1738,7 @@
         <v>35</v>
       </c>
       <c r="D30" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="E30" t="s">
         <v>41</v>
@@ -1877,7 +1896,7 @@
         <v>17</v>
       </c>
       <c r="G6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -1917,7 +1936,7 @@
         <v>28</v>
       </c>
       <c r="G8" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -1931,7 +1950,7 @@
         <v>29</v>
       </c>
       <c r="G9" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Added icons and full body image compatibility
</commit_message>
<xml_diff>
--- a/TrailsTimeline.xlsx
+++ b/TrailsTimeline.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6da5a9201bc5826c/Documentos/trails_orbal_atlas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="13_ncr:1_{54315043-5A41-45C0-BA2E-F1BBE0C76030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B644D1B2-3E0C-4C83-888F-355B1550FBC7}"/>
+  <xr:revisionPtr revIDLastSave="51" documentId="13_ncr:1_{54315043-5A41-45C0-BA2E-F1BBE0C76030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2E6D6F28-ED43-4AC4-8325-A29B98D95FDF}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{B6393BEF-99C0-4DAE-AD63-40B518CD1F0D}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="136">
   <si>
     <t>char_id</t>
   </si>
@@ -400,6 +400,57 @@
   </si>
   <si>
     <t>reveal_name</t>
+  </si>
+  <si>
+    <t>weismann1.webp</t>
+  </si>
+  <si>
+    <t>weismannFullBody1.webp</t>
+  </si>
+  <si>
+    <t>cassius1.png</t>
+  </si>
+  <si>
+    <t>cassiusFullBody1.png</t>
+  </si>
+  <si>
+    <t>josetteCapua1.png</t>
+  </si>
+  <si>
+    <t>josetteFullBody1.webp</t>
+  </si>
+  <si>
+    <t>estelle1.png</t>
+  </si>
+  <si>
+    <t>joshua1.png</t>
+  </si>
+  <si>
+    <t>estelleFullBody1.webp</t>
+  </si>
+  <si>
+    <t>joshuaFullBody1.png</t>
+  </si>
+  <si>
+    <t>scherazard1.webp</t>
+  </si>
+  <si>
+    <t>scherazardFullBody1.webp</t>
+  </si>
+  <si>
+    <t>josetteCapua2.png</t>
+  </si>
+  <si>
+    <t>josetterFullBody2.png</t>
+  </si>
+  <si>
+    <t>Estelle's and Joshua's bracer mentor</t>
+  </si>
+  <si>
+    <t>Adopted brother of Estelle</t>
+  </si>
+  <si>
+    <t>Her mother died protecting her during the 100 day war</t>
   </si>
 </sst>
 </file>
@@ -788,7 +839,8 @@
     <col min="3" max="3" width="19.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="20.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="4.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -830,6 +882,12 @@
       <c r="E2" t="s">
         <v>34</v>
       </c>
+      <c r="F2" t="s">
+        <v>125</v>
+      </c>
+      <c r="G2" t="s">
+        <v>127</v>
+      </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
@@ -847,6 +905,12 @@
       <c r="E3" t="s">
         <v>34</v>
       </c>
+      <c r="F3" t="s">
+        <v>126</v>
+      </c>
+      <c r="G3" t="s">
+        <v>128</v>
+      </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
@@ -864,6 +928,12 @@
       <c r="E4" t="s">
         <v>34</v>
       </c>
+      <c r="F4" t="s">
+        <v>129</v>
+      </c>
+      <c r="G4" t="s">
+        <v>130</v>
+      </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
@@ -881,6 +951,12 @@
       <c r="E5" t="s">
         <v>34</v>
       </c>
+      <c r="F5" t="s">
+        <v>121</v>
+      </c>
+      <c r="G5" t="s">
+        <v>122</v>
+      </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
@@ -898,6 +974,12 @@
       <c r="E6" t="s">
         <v>34</v>
       </c>
+      <c r="F6" t="s">
+        <v>123</v>
+      </c>
+      <c r="G6" t="s">
+        <v>124</v>
+      </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
@@ -914,6 +996,12 @@
       </c>
       <c r="E7" t="s">
         <v>34</v>
+      </c>
+      <c r="F7" t="s">
+        <v>119</v>
+      </c>
+      <c r="G7" t="s">
+        <v>120</v>
       </c>
     </row>
   </sheetData>
@@ -1992,13 +2080,16 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76C493BF-D343-46EF-AB39-E5F4461CCFFF}">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="15.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15.85546875" customWidth="1"/>
     <col min="4" max="4" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="29.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="48.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2043,6 +2134,12 @@
       <c r="E2" t="s">
         <v>53</v>
       </c>
+      <c r="G2" t="s">
+        <v>131</v>
+      </c>
+      <c r="H2" t="s">
+        <v>132</v>
+      </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
@@ -2076,6 +2173,57 @@
       </c>
       <c r="E4" t="s">
         <v>83</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C5">
+        <v>12</v>
+      </c>
+      <c r="D5" t="s">
+        <v>56</v>
+      </c>
+      <c r="E5" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" t="s">
+        <v>34</v>
+      </c>
+      <c r="C6">
+        <v>10</v>
+      </c>
+      <c r="D6" t="s">
+        <v>56</v>
+      </c>
+      <c r="E6" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>34</v>
+      </c>
+      <c r="C7">
+        <v>10</v>
+      </c>
+      <c r="D7" t="s">
+        <v>56</v>
+      </c>
+      <c r="E7" t="s">
+        <v>135</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated data to add image roots
</commit_message>
<xml_diff>
--- a/TrailsTimeline.xlsx
+++ b/TrailsTimeline.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6da5a9201bc5826c/Documentos/trails_orbal_atlas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="51" documentId="13_ncr:1_{54315043-5A41-45C0-BA2E-F1BBE0C76030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2E6D6F28-ED43-4AC4-8325-A29B98D95FDF}"/>
+  <xr:revisionPtr revIDLastSave="53" documentId="13_ncr:1_{54315043-5A41-45C0-BA2E-F1BBE0C76030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7610CD3D-53A8-446F-8A2A-9AF724C858F7}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{B6393BEF-99C0-4DAE-AD63-40B518CD1F0D}"/>
   </bookViews>
@@ -2120,110 +2120,110 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>44</v>
+        <v>10</v>
       </c>
       <c r="B2" t="s">
         <v>34</v>
       </c>
       <c r="C2">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="D2" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="E2" t="s">
-        <v>53</v>
-      </c>
-      <c r="G2" t="s">
-        <v>131</v>
-      </c>
-      <c r="H2" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>44</v>
+        <v>6</v>
       </c>
       <c r="B3" t="s">
         <v>34</v>
       </c>
       <c r="C3">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="D3" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E3" t="s">
-        <v>54</v>
+        <v>135</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B4" t="s">
         <v>34</v>
       </c>
       <c r="C4">
-        <v>38</v>
+        <v>12</v>
       </c>
       <c r="D4" t="s">
         <v>56</v>
       </c>
       <c r="E4" t="s">
-        <v>83</v>
+        <v>133</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>12</v>
+        <v>44</v>
       </c>
       <c r="B5" t="s">
         <v>34</v>
       </c>
       <c r="C5">
-        <v>12</v>
+        <v>32</v>
       </c>
       <c r="D5" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="E5" t="s">
-        <v>133</v>
+        <v>53</v>
+      </c>
+      <c r="G5" t="s">
+        <v>131</v>
+      </c>
+      <c r="H5" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>44</v>
       </c>
       <c r="B6" t="s">
         <v>34</v>
       </c>
       <c r="C6">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="D6" t="s">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="E6" t="s">
-        <v>134</v>
+        <v>54</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="B7" t="s">
         <v>34</v>
       </c>
       <c r="C7">
-        <v>10</v>
+        <v>38</v>
       </c>
       <c r="D7" t="s">
         <v>56</v>
       </c>
       <c r="E7" t="s">
-        <v>135</v>
+        <v>83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Corrected cassius appearances and josette's first full body image
</commit_message>
<xml_diff>
--- a/TrailsTimeline.xlsx
+++ b/TrailsTimeline.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6da5a9201bc5826c/Documentos/trails_orbal_atlas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="53" documentId="13_ncr:1_{54315043-5A41-45C0-BA2E-F1BBE0C76030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7610CD3D-53A8-446F-8A2A-9AF724C858F7}"/>
+  <xr:revisionPtr revIDLastSave="57" documentId="13_ncr:1_{54315043-5A41-45C0-BA2E-F1BBE0C76030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E62596D7-D619-4697-B0AC-0945D669D5CE}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{B6393BEF-99C0-4DAE-AD63-40B518CD1F0D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B6393BEF-99C0-4DAE-AD63-40B518CD1F0D}"/>
   </bookViews>
   <sheets>
     <sheet name="characters" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="136">
   <si>
     <t>char_id</t>
   </si>
@@ -441,9 +441,6 @@
     <t>josetteCapua2.png</t>
   </si>
   <si>
-    <t>josetterFullBody2.png</t>
-  </si>
-  <si>
     <t>Estelle's and Joshua's bracer mentor</t>
   </si>
   <si>
@@ -451,6 +448,9 @@
   </si>
   <si>
     <t>Her mother died protecting her during the 100 day war</t>
+  </si>
+  <si>
+    <t>josetteFullBody2.png</t>
   </si>
 </sst>
 </file>
@@ -1943,14 +1943,11 @@
       <c r="C4">
         <v>10</v>
       </c>
-      <c r="D4" t="s">
-        <v>41</v>
-      </c>
       <c r="E4" t="s">
         <v>34</v>
       </c>
       <c r="F4">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G4" t="s">
         <v>64</v>
@@ -1990,7 +1987,7 @@
         <v>34</v>
       </c>
       <c r="F6">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G6" t="s">
         <v>112</v>
@@ -2132,7 +2129,7 @@
         <v>56</v>
       </c>
       <c r="E2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -2149,7 +2146,7 @@
         <v>56</v>
       </c>
       <c r="E3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -2166,7 +2163,7 @@
         <v>56</v>
       </c>
       <c r="E4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -2189,7 +2186,7 @@
         <v>131</v>
       </c>
       <c r="H5" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
corrected how icons are displayed on map
</commit_message>
<xml_diff>
--- a/TrailsTimeline.xlsx
+++ b/TrailsTimeline.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6da5a9201bc5826c/Documentos/trails_orbal_atlas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="57" documentId="13_ncr:1_{54315043-5A41-45C0-BA2E-F1BBE0C76030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E62596D7-D619-4697-B0AC-0945D669D5CE}"/>
+  <xr:revisionPtr revIDLastSave="63" documentId="13_ncr:1_{54315043-5A41-45C0-BA2E-F1BBE0C76030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B140CF64-9ADF-4D7A-93A2-152A5B3FEB82}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B6393BEF-99C0-4DAE-AD63-40B518CD1F0D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{B6393BEF-99C0-4DAE-AD63-40B518CD1F0D}"/>
   </bookViews>
   <sheets>
     <sheet name="characters" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="137">
   <si>
     <t>char_id</t>
   </si>
@@ -451,6 +451,9 @@
   </si>
   <si>
     <t>josetteFullBody2.png</t>
+  </si>
+  <si>
+    <t>Anthropologist investigating the Tetracyclic towers</t>
   </si>
 </sst>
 </file>
@@ -2077,7 +2080,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76C493BF-D343-46EF-AB39-E5F4461CCFFF}">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="15.85546875" bestFit="1" customWidth="1"/>
@@ -2168,25 +2171,19 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>44</v>
+        <v>96</v>
       </c>
       <c r="B5" t="s">
         <v>34</v>
       </c>
       <c r="C5">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="D5" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="E5" t="s">
-        <v>53</v>
-      </c>
-      <c r="G5" t="s">
-        <v>131</v>
-      </c>
-      <c r="H5" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -2200,26 +2197,49 @@
         <v>32</v>
       </c>
       <c r="D6" t="s">
-        <v>2</v>
+        <v>52</v>
       </c>
       <c r="E6" t="s">
-        <v>54</v>
+        <v>53</v>
+      </c>
+      <c r="G6" t="s">
+        <v>131</v>
+      </c>
+      <c r="H6" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>44</v>
+      </c>
+      <c r="B7" t="s">
+        <v>34</v>
+      </c>
+      <c r="C7">
+        <v>32</v>
+      </c>
+      <c r="D7" t="s">
+        <v>2</v>
+      </c>
+      <c r="E7" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>14</v>
       </c>
-      <c r="B7" t="s">
-        <v>34</v>
-      </c>
-      <c r="C7">
+      <c r="B8" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8">
         <v>38</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D8" t="s">
         <v>56</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E8" t="s">
         <v>83</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Corrected map icon display
</commit_message>
<xml_diff>
--- a/TrailsTimeline.xlsx
+++ b/TrailsTimeline.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6da5a9201bc5826c/Documentos/trails_orbal_atlas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="63" documentId="13_ncr:1_{54315043-5A41-45C0-BA2E-F1BBE0C76030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B140CF64-9ADF-4D7A-93A2-152A5B3FEB82}"/>
+  <xr:revisionPtr revIDLastSave="70" documentId="13_ncr:1_{54315043-5A41-45C0-BA2E-F1BBE0C76030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BA530130-0C14-4E88-AD8E-A8EF42AECBFC}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{B6393BEF-99C0-4DAE-AD63-40B518CD1F0D}"/>
   </bookViews>
@@ -294,9 +294,6 @@
     <t>Bose City</t>
   </si>
   <si>
-    <t>Disappeared on captured airliner</t>
-  </si>
-  <si>
     <t>Party leader</t>
   </si>
   <si>
@@ -441,19 +438,22 @@
     <t>josetteCapua2.png</t>
   </si>
   <si>
-    <t>Estelle's and Joshua's bracer mentor</t>
-  </si>
-  <si>
-    <t>Adopted brother of Estelle</t>
-  </si>
-  <si>
-    <t>Her mother died protecting her during the 100 day war</t>
-  </si>
-  <si>
     <t>josetteFullBody2.png</t>
   </si>
   <si>
-    <t>Anthropologist investigating the Tetracyclic towers</t>
+    <t>Adopted brother of Estelle.</t>
+  </si>
+  <si>
+    <t>Her mother died protecting her during the 100 day war.</t>
+  </si>
+  <si>
+    <t>Archeologist investigating the Tetracyclic towers.</t>
+  </si>
+  <si>
+    <t>Bracer mentor for Estelle and Joshua.</t>
+  </si>
+  <si>
+    <t>Disappeared on captured airliner.</t>
   </si>
 </sst>
 </file>
@@ -866,7 +866,7 @@
         <v>5</v>
       </c>
       <c r="G1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -886,10 +886,10 @@
         <v>34</v>
       </c>
       <c r="F2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="G2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -909,10 +909,10 @@
         <v>34</v>
       </c>
       <c r="F3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -932,10 +932,10 @@
         <v>34</v>
       </c>
       <c r="F4" t="s">
+        <v>128</v>
+      </c>
+      <c r="G4" t="s">
         <v>129</v>
-      </c>
-      <c r="G4" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -955,10 +955,10 @@
         <v>34</v>
       </c>
       <c r="F5" t="s">
+        <v>120</v>
+      </c>
+      <c r="G5" t="s">
         <v>121</v>
-      </c>
-      <c r="G5" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -978,21 +978,21 @@
         <v>34</v>
       </c>
       <c r="F6" t="s">
+        <v>122</v>
+      </c>
+      <c r="G6" t="s">
         <v>123</v>
-      </c>
-      <c r="G6" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>95</v>
+      </c>
+      <c r="B7" t="s">
         <v>96</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>97</v>
-      </c>
-      <c r="C7" t="s">
-        <v>98</v>
       </c>
       <c r="D7" t="s">
         <v>39</v>
@@ -1001,10 +1001,10 @@
         <v>34</v>
       </c>
       <c r="F7" t="s">
+        <v>118</v>
+      </c>
+      <c r="G7" t="s">
         <v>119</v>
-      </c>
-      <c r="G7" t="s">
-        <v>120</v>
       </c>
     </row>
   </sheetData>
@@ -1041,7 +1041,7 @@
         <v>21</v>
       </c>
       <c r="G1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -1278,7 +1278,7 @@
         <v>35</v>
       </c>
       <c r="D2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E2" t="s">
         <v>41</v>
@@ -1318,7 +1318,7 @@
         <v>35</v>
       </c>
       <c r="D4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E4" t="s">
         <v>79</v>
@@ -1338,7 +1338,7 @@
         <v>35</v>
       </c>
       <c r="D5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E5" t="s">
         <v>79</v>
@@ -1358,7 +1358,7 @@
         <v>35</v>
       </c>
       <c r="D6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E6" t="s">
         <v>39</v>
@@ -1398,7 +1398,7 @@
         <v>35</v>
       </c>
       <c r="D8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E8" t="s">
         <v>41</v>
@@ -1418,7 +1418,7 @@
         <v>35</v>
       </c>
       <c r="D9" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E9" t="s">
         <v>37</v>
@@ -1438,7 +1438,7 @@
         <v>35</v>
       </c>
       <c r="D10" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E10" t="s">
         <v>37</v>
@@ -1478,7 +1478,7 @@
         <v>35</v>
       </c>
       <c r="D12" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E12" t="s">
         <v>79</v>
@@ -1498,7 +1498,7 @@
         <v>35</v>
       </c>
       <c r="D13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E13" t="s">
         <v>42</v>
@@ -1518,7 +1518,7 @@
         <v>35</v>
       </c>
       <c r="D14" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E14" t="s">
         <v>42</v>
@@ -1558,7 +1558,7 @@
         <v>35</v>
       </c>
       <c r="D16" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E16" t="s">
         <v>79</v>
@@ -1578,7 +1578,7 @@
         <v>35</v>
       </c>
       <c r="D17" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E17" t="s">
         <v>79</v>
@@ -1598,7 +1598,7 @@
         <v>35</v>
       </c>
       <c r="D18" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E18" t="s">
         <v>39</v>
@@ -1618,7 +1618,7 @@
         <v>35</v>
       </c>
       <c r="D19" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E19" t="s">
         <v>39</v>
@@ -1638,7 +1638,7 @@
         <v>35</v>
       </c>
       <c r="D20" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E20" t="s">
         <v>79</v>
@@ -1658,7 +1658,7 @@
         <v>35</v>
       </c>
       <c r="D21" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E21" t="s">
         <v>79</v>
@@ -1678,7 +1678,7 @@
         <v>35</v>
       </c>
       <c r="D22" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E22" t="s">
         <v>79</v>
@@ -1718,7 +1718,7 @@
         <v>35</v>
       </c>
       <c r="D24" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E24" t="s">
         <v>47</v>
@@ -1738,7 +1738,7 @@
         <v>35</v>
       </c>
       <c r="D25" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E25" t="s">
         <v>47</v>
@@ -1758,7 +1758,7 @@
         <v>35</v>
       </c>
       <c r="D26" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E26" t="s">
         <v>47</v>
@@ -1778,7 +1778,7 @@
         <v>35</v>
       </c>
       <c r="D27" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E27" t="s">
         <v>79</v>
@@ -1798,7 +1798,7 @@
         <v>35</v>
       </c>
       <c r="D28" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E28" t="s">
         <v>79</v>
@@ -1818,7 +1818,7 @@
         <v>35</v>
       </c>
       <c r="D29" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E29" t="s">
         <v>41</v>
@@ -1838,7 +1838,7 @@
         <v>35</v>
       </c>
       <c r="D30" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E30" t="s">
         <v>41</v>
@@ -1919,7 +1919,7 @@
         <v>10</v>
       </c>
       <c r="G2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -1933,7 +1933,7 @@
         <v>10</v>
       </c>
       <c r="G3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -1973,7 +1973,7 @@
         <v>13</v>
       </c>
       <c r="G5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -1993,7 +1993,7 @@
         <v>16</v>
       </c>
       <c r="G6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -2018,7 +2018,7 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B8" t="s">
         <v>34</v>
@@ -2033,7 +2033,7 @@
         <v>28</v>
       </c>
       <c r="G8" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -2047,7 +2047,7 @@
         <v>29</v>
       </c>
       <c r="G9" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -2109,13 +2109,13 @@
         <v>51</v>
       </c>
       <c r="F1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G1" t="s">
         <v>5</v>
       </c>
       <c r="H1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -2132,7 +2132,7 @@
         <v>56</v>
       </c>
       <c r="E2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -2149,7 +2149,7 @@
         <v>56</v>
       </c>
       <c r="E3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -2166,12 +2166,12 @@
         <v>56</v>
       </c>
       <c r="E4" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B5" t="s">
         <v>34</v>
@@ -2183,7 +2183,7 @@
         <v>56</v>
       </c>
       <c r="E5" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -2203,10 +2203,10 @@
         <v>53</v>
       </c>
       <c r="G6" t="s">
+        <v>130</v>
+      </c>
+      <c r="H6" t="s">
         <v>131</v>
-      </c>
-      <c r="H6" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -2240,7 +2240,7 @@
         <v>56</v>
       </c>
       <c r="E8" t="s">
-        <v>83</v>
+        <v>136</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated bio behavior and data
</commit_message>
<xml_diff>
--- a/TrailsTimeline.xlsx
+++ b/TrailsTimeline.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6da5a9201bc5826c/Documentos/trails_orbal_atlas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="70" documentId="13_ncr:1_{54315043-5A41-45C0-BA2E-F1BBE0C76030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BA530130-0C14-4E88-AD8E-A8EF42AECBFC}"/>
+  <xr:revisionPtr revIDLastSave="175" documentId="13_ncr:1_{54315043-5A41-45C0-BA2E-F1BBE0C76030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{15309D8E-A697-4A6F-A2E5-845D57CE9B2C}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{B6393BEF-99C0-4DAE-AD63-40B518CD1F0D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{B6393BEF-99C0-4DAE-AD63-40B518CD1F0D}"/>
   </bookViews>
   <sheets>
     <sheet name="characters" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="144">
   <si>
     <t>char_id</t>
   </si>
@@ -201,9 +201,6 @@
     <t>text</t>
   </si>
   <si>
-    <t>identity</t>
-  </si>
-  <si>
     <t>Josette Capua</t>
   </si>
   <si>
@@ -321,12 +318,6 @@
     <t>Rescuing miners from a cave in and recovering crystal</t>
   </si>
   <si>
-    <t>Rescuing children from Esmelas Tower</t>
-  </si>
-  <si>
-    <t>Learning about Septium crystal that needs retrieving from Mayor Klaus</t>
-  </si>
-  <si>
     <t>Delivering crystal to Mayor Klaus, encountering Josette</t>
   </si>
   <si>
@@ -441,19 +432,49 @@
     <t>josetteFullBody2.png</t>
   </si>
   <si>
-    <t>Adopted brother of Estelle.</t>
-  </si>
-  <si>
-    <t>Her mother died protecting her during the 100 day war.</t>
-  </si>
-  <si>
-    <t>Archeologist investigating the Tetracyclic towers.</t>
-  </si>
-  <si>
-    <t>Bracer mentor for Estelle and Joshua.</t>
-  </si>
-  <si>
-    <t>Disappeared on captured airliner.</t>
+    <t>Attempting to rescue children from Esmelas Tower</t>
+  </si>
+  <si>
+    <t>Ambushed by monsters, Cassius comes to the rescue</t>
+  </si>
+  <si>
+    <t>On a work trip with the Bracer Guild</t>
+  </si>
+  <si>
+    <t>Attempted to steal the Esmelas Crystal that was going to be gifted to the Queen</t>
+  </si>
+  <si>
+    <t>Doing the easier of the bracer jobs left over by Cassius with Joshua</t>
+  </si>
+  <si>
+    <t>Doing the easier of the bracer jobs left over by Cassius with Estelle</t>
+  </si>
+  <si>
+    <t>Doing the hardest of the bracer jobs left by Cassius</t>
+  </si>
+  <si>
+    <t>Accompanying Estelle and Joshua to Bose on their search for Cassius</t>
+  </si>
+  <si>
+    <t>Adopted brother of Estelle</t>
+  </si>
+  <si>
+    <t>Her mother died protecting her during the 100 day war</t>
+  </si>
+  <si>
+    <t>Bracer mentor for Estelle and Joshua</t>
+  </si>
+  <si>
+    <t>S rank Bracer</t>
+  </si>
+  <si>
+    <t>Archeologist investigating the Tetracyclic towers</t>
+  </si>
+  <si>
+    <t>Disappeared on captured airliner</t>
+  </si>
+  <si>
+    <t>Learning about Esmelas Crystal that needs retrieving from Mayor Klaus</t>
   </si>
 </sst>
 </file>
@@ -866,7 +887,7 @@
         <v>5</v>
       </c>
       <c r="G1" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -886,10 +907,10 @@
         <v>34</v>
       </c>
       <c r="F2" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="G2" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -909,10 +930,10 @@
         <v>34</v>
       </c>
       <c r="F3" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="G3" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -926,16 +947,16 @@
         <v>8</v>
       </c>
       <c r="D4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E4" t="s">
         <v>34</v>
       </c>
       <c r="F4" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="G4" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -955,10 +976,10 @@
         <v>34</v>
       </c>
       <c r="F5" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="G5" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -972,27 +993,27 @@
         <v>46</v>
       </c>
       <c r="D6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E6" t="s">
         <v>34</v>
       </c>
       <c r="F6" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G6" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="B7" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="C7" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="D7" t="s">
         <v>39</v>
@@ -1001,10 +1022,10 @@
         <v>34</v>
       </c>
       <c r="F7" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="G7" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
     </row>
   </sheetData>
@@ -1041,7 +1062,7 @@
         <v>21</v>
       </c>
       <c r="G1" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -1055,15 +1076,15 @@
         <v>23</v>
       </c>
       <c r="D2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B3" t="s">
         <v>79</v>
-      </c>
-      <c r="B3" t="s">
-        <v>80</v>
       </c>
       <c r="C3" t="s">
         <v>9</v>
@@ -1094,7 +1115,7 @@
         <v>39</v>
       </c>
       <c r="B5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C5" t="s">
         <v>9</v>
@@ -1137,7 +1158,7 @@
         <v>41</v>
       </c>
       <c r="B7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C7" t="s">
         <v>9</v>
@@ -1200,27 +1221,27 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B10" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C10" t="s">
         <v>23</v>
       </c>
       <c r="D10" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>80</v>
+      </c>
+      <c r="B11" t="s">
         <v>81</v>
       </c>
-      <c r="B11" t="s">
-        <v>82</v>
-      </c>
       <c r="C11" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D11" t="s">
         <v>24</v>
@@ -1239,7 +1260,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{94EA2C8E-D265-418D-8065-F972E277CAB9}">
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="78.5703125" bestFit="1" customWidth="1"/>
@@ -1278,7 +1299,7 @@
         <v>35</v>
       </c>
       <c r="D2" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="E2" t="s">
         <v>41</v>
@@ -1301,7 +1322,7 @@
         <v>36</v>
       </c>
       <c r="E3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F3" t="s">
         <v>33</v>
@@ -1318,10 +1339,10 @@
         <v>35</v>
       </c>
       <c r="D4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F4" t="s">
         <v>33</v>
@@ -1338,10 +1359,10 @@
         <v>35</v>
       </c>
       <c r="D5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F5" t="s">
         <v>33</v>
@@ -1358,7 +1379,7 @@
         <v>35</v>
       </c>
       <c r="D6" t="s">
-        <v>92</v>
+        <v>129</v>
       </c>
       <c r="E6" t="s">
         <v>39</v>
@@ -1378,10 +1399,10 @@
         <v>35</v>
       </c>
       <c r="D7" t="s">
-        <v>71</v>
+        <v>130</v>
       </c>
       <c r="E7" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F7" t="s">
         <v>33</v>
@@ -1398,7 +1419,7 @@
         <v>35</v>
       </c>
       <c r="D8" t="s">
-        <v>89</v>
+        <v>70</v>
       </c>
       <c r="E8" t="s">
         <v>41</v>
@@ -1418,13 +1439,13 @@
         <v>35</v>
       </c>
       <c r="D9" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E9" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="F9" t="s">
-        <v>73</v>
+        <v>33</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -1438,13 +1459,13 @@
         <v>35</v>
       </c>
       <c r="D10" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="E10" t="s">
         <v>37</v>
       </c>
       <c r="F10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -1458,13 +1479,13 @@
         <v>35</v>
       </c>
       <c r="D11" t="s">
+        <v>87</v>
+      </c>
+      <c r="E11" t="s">
+        <v>37</v>
+      </c>
+      <c r="F11" t="s">
         <v>72</v>
-      </c>
-      <c r="E11" t="s">
-        <v>79</v>
-      </c>
-      <c r="F11" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -1478,13 +1499,13 @@
         <v>35</v>
       </c>
       <c r="D12" t="s">
-        <v>93</v>
+        <v>71</v>
       </c>
       <c r="E12" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F12" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -1498,13 +1519,13 @@
         <v>35</v>
       </c>
       <c r="D13" t="s">
-        <v>90</v>
+        <v>143</v>
       </c>
       <c r="E13" t="s">
-        <v>42</v>
+        <v>78</v>
       </c>
       <c r="F13" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -1518,13 +1539,13 @@
         <v>35</v>
       </c>
       <c r="D14" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E14" t="s">
         <v>42</v>
       </c>
       <c r="F14" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -1538,13 +1559,13 @@
         <v>35</v>
       </c>
       <c r="D15" t="s">
+        <v>90</v>
+      </c>
+      <c r="E15" t="s">
+        <v>42</v>
+      </c>
+      <c r="F15" t="s">
         <v>72</v>
-      </c>
-      <c r="E15" t="s">
-        <v>79</v>
-      </c>
-      <c r="F15" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -1558,13 +1579,13 @@
         <v>35</v>
       </c>
       <c r="D16" t="s">
-        <v>94</v>
+        <v>71</v>
       </c>
       <c r="E16" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F16" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
@@ -1578,13 +1599,13 @@
         <v>35</v>
       </c>
       <c r="D17" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="E17" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F17" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
@@ -1598,13 +1619,13 @@
         <v>35</v>
       </c>
       <c r="D18" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="E18" t="s">
-        <v>39</v>
+        <v>78</v>
       </c>
       <c r="F18" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
@@ -1618,13 +1639,13 @@
         <v>35</v>
       </c>
       <c r="D19" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E19" t="s">
         <v>39</v>
       </c>
       <c r="F19" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
@@ -1638,13 +1659,13 @@
         <v>35</v>
       </c>
       <c r="D20" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="E20" t="s">
-        <v>79</v>
+        <v>39</v>
       </c>
       <c r="F20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
@@ -1658,13 +1679,13 @@
         <v>35</v>
       </c>
       <c r="D21" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="E21" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F21" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
@@ -1678,13 +1699,13 @@
         <v>35</v>
       </c>
       <c r="D22" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="E22" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F22" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
@@ -1698,13 +1719,13 @@
         <v>35</v>
       </c>
       <c r="D23" t="s">
-        <v>63</v>
+        <v>100</v>
       </c>
       <c r="E23" t="s">
-        <v>47</v>
+        <v>78</v>
       </c>
       <c r="F23" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
@@ -1718,13 +1739,13 @@
         <v>35</v>
       </c>
       <c r="D24" t="s">
-        <v>104</v>
+        <v>62</v>
       </c>
       <c r="E24" t="s">
         <v>47</v>
       </c>
       <c r="F24" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
@@ -1738,13 +1759,13 @@
         <v>35</v>
       </c>
       <c r="D25" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="E25" t="s">
         <v>47</v>
       </c>
       <c r="F25" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
@@ -1758,13 +1779,13 @@
         <v>35</v>
       </c>
       <c r="D26" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="E26" t="s">
         <v>47</v>
       </c>
       <c r="F26" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
@@ -1778,13 +1799,13 @@
         <v>35</v>
       </c>
       <c r="D27" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="E27" t="s">
-        <v>79</v>
+        <v>47</v>
       </c>
       <c r="F27" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
@@ -1798,13 +1819,13 @@
         <v>35</v>
       </c>
       <c r="D28" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="E28" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F28" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
@@ -1818,13 +1839,13 @@
         <v>35</v>
       </c>
       <c r="D29" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="E29" t="s">
-        <v>41</v>
+        <v>78</v>
       </c>
       <c r="F29" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
@@ -1838,33 +1859,53 @@
         <v>35</v>
       </c>
       <c r="D30" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="E30" t="s">
         <v>41</v>
       </c>
       <c r="F30" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
+        <v>34</v>
+      </c>
+      <c r="B31">
+        <v>39</v>
+      </c>
+      <c r="C31" t="s">
+        <v>35</v>
+      </c>
+      <c r="D31" t="s">
+        <v>111</v>
+      </c>
+      <c r="E31" t="s">
+        <v>41</v>
+      </c>
+      <c r="F31" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>67</v>
+      </c>
+      <c r="B32">
+        <v>50</v>
+      </c>
+      <c r="C32" t="s">
         <v>68</v>
       </c>
-      <c r="B31">
-        <v>50</v>
-      </c>
-      <c r="C31" t="s">
+      <c r="D32" t="s">
+        <v>76</v>
+      </c>
+      <c r="E32" t="s">
+        <v>80</v>
+      </c>
+      <c r="F32" t="s">
         <v>69</v>
-      </c>
-      <c r="D31" t="s">
-        <v>77</v>
-      </c>
-      <c r="E31" t="s">
-        <v>81</v>
-      </c>
-      <c r="F31" t="s">
-        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -1890,22 +1931,22 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1" t="s">
         <v>57</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>58</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>59</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>60</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>61</v>
-      </c>
-      <c r="G1" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -1916,10 +1957,11 @@
         <v>34</v>
       </c>
       <c r="C2">
+        <f>beats!B2</f>
         <v>10</v>
       </c>
       <c r="G2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -1930,10 +1972,11 @@
         <v>34</v>
       </c>
       <c r="C3">
+        <f>beats!B2</f>
         <v>10</v>
       </c>
       <c r="G3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -1944,16 +1987,18 @@
         <v>34</v>
       </c>
       <c r="C4">
+        <f>beats!B2</f>
         <v>10</v>
       </c>
       <c r="E4" t="s">
         <v>34</v>
       </c>
       <c r="F4">
+        <f>beats!B2</f>
         <v>10</v>
       </c>
       <c r="G4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -1964,16 +2009,18 @@
         <v>34</v>
       </c>
       <c r="C5">
+        <f>beats!B3</f>
         <v>11</v>
       </c>
       <c r="E5" t="s">
         <v>34</v>
       </c>
       <c r="F5">
+        <f>beats!B5</f>
         <v>13</v>
       </c>
       <c r="G5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -1984,16 +2031,18 @@
         <v>34</v>
       </c>
       <c r="C6">
-        <v>14</v>
+        <f>beats!B7</f>
+        <v>15</v>
       </c>
       <c r="E6" t="s">
         <v>34</v>
       </c>
       <c r="F6">
-        <v>16</v>
+        <f>beats!B9</f>
+        <v>17</v>
       </c>
       <c r="G6" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -2004,36 +2053,40 @@
         <v>34</v>
       </c>
       <c r="C7">
-        <v>24</v>
+        <f>beats!B17</f>
+        <v>25</v>
       </c>
       <c r="E7" t="s">
         <v>34</v>
       </c>
       <c r="F7">
-        <v>25</v>
+        <f>beats!B18</f>
+        <v>26</v>
       </c>
       <c r="G7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="B8" t="s">
         <v>34</v>
       </c>
       <c r="C8">
-        <v>27</v>
+        <f>beats!B20</f>
+        <v>28</v>
       </c>
       <c r="E8" t="s">
         <v>34</v>
       </c>
       <c r="F8">
-        <v>28</v>
+        <f>beats!B21</f>
+        <v>29</v>
       </c>
       <c r="G8" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -2044,10 +2097,11 @@
         <v>34</v>
       </c>
       <c r="C9">
-        <v>29</v>
+        <f>beats!B22</f>
+        <v>30</v>
       </c>
       <c r="G9" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -2058,7 +2112,8 @@
         <v>34</v>
       </c>
       <c r="C10">
-        <v>32</v>
+        <f>beats!B25</f>
+        <v>33</v>
       </c>
       <c r="D10" t="s">
         <v>47</v>
@@ -2067,10 +2122,11 @@
         <v>34</v>
       </c>
       <c r="F10">
-        <v>34</v>
+        <f>beats!B27</f>
+        <v>35</v>
       </c>
       <c r="G10" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
   </sheetData>
@@ -2080,14 +2136,14 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76C493BF-D343-46EF-AB39-E5F4461CCFFF}">
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="15.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15.85546875" customWidth="1"/>
     <col min="4" max="4" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="48.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="70.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.28515625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="19.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="20.28515625" bestFit="1" customWidth="1"/>
   </cols>
@@ -2109,13 +2165,13 @@
         <v>51</v>
       </c>
       <c r="F1" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="G1" t="s">
         <v>5</v>
       </c>
       <c r="H1" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -2126,13 +2182,14 @@
         <v>34</v>
       </c>
       <c r="C2">
+        <f>beats!B2</f>
         <v>10</v>
       </c>
       <c r="D2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E2" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -2143,13 +2200,14 @@
         <v>34</v>
       </c>
       <c r="C3">
+        <f>beats!B2</f>
         <v>10</v>
       </c>
       <c r="D3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E3" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -2160,86 +2218,238 @@
         <v>34</v>
       </c>
       <c r="C4">
+        <f>beats!B4</f>
         <v>12</v>
       </c>
       <c r="D4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E4" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>95</v>
+        <v>14</v>
       </c>
       <c r="B5" t="s">
         <v>34</v>
       </c>
       <c r="C5">
-        <v>27</v>
+        <f>beats!B9</f>
+        <v>17</v>
       </c>
       <c r="D5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E5" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="B6" t="s">
         <v>34</v>
       </c>
       <c r="C6">
-        <v>32</v>
+        <f>beats!B9</f>
+        <v>17</v>
       </c>
       <c r="D6" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="E6" t="s">
-        <v>53</v>
-      </c>
-      <c r="G6" t="s">
-        <v>130</v>
-      </c>
-      <c r="H6" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>44</v>
+        <v>6</v>
       </c>
       <c r="B7" t="s">
         <v>34</v>
       </c>
       <c r="C7">
-        <v>32</v>
+        <f>beats!B9</f>
+        <v>17</v>
       </c>
       <c r="D7" t="s">
-        <v>2</v>
+        <v>55</v>
       </c>
       <c r="E7" t="s">
-        <v>54</v>
+        <v>133</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8">
+        <f>beats!B9</f>
+        <v>17</v>
+      </c>
+      <c r="D8" t="s">
+        <v>55</v>
+      </c>
+      <c r="E8" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" t="s">
+        <v>34</v>
+      </c>
+      <c r="C9">
+        <f>beats!B9</f>
+        <v>17</v>
+      </c>
+      <c r="D9" t="s">
+        <v>55</v>
+      </c>
+      <c r="E9" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>92</v>
+      </c>
+      <c r="B10" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10">
+        <f>beats!B19</f>
+        <v>27</v>
+      </c>
+      <c r="D10" t="s">
+        <v>55</v>
+      </c>
+      <c r="E10" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>44</v>
+      </c>
+      <c r="B11" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11">
+        <f>beats!B24</f>
+        <v>32</v>
+      </c>
+      <c r="D11" t="s">
+        <v>55</v>
+      </c>
+      <c r="E11" t="s">
+        <v>132</v>
+      </c>
+      <c r="F11" t="s">
+        <v>52</v>
+      </c>
+      <c r="G11" t="s">
+        <v>127</v>
+      </c>
+      <c r="H11" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>44</v>
+      </c>
+      <c r="B12" t="s">
+        <v>34</v>
+      </c>
+      <c r="C12">
+        <f>beats!B24</f>
+        <v>32</v>
+      </c>
+      <c r="D12" t="s">
+        <v>2</v>
+      </c>
+      <c r="E12" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>14</v>
       </c>
-      <c r="B8" t="s">
-        <v>34</v>
-      </c>
-      <c r="C8">
+      <c r="B13" t="s">
+        <v>34</v>
+      </c>
+      <c r="C13">
+        <f>beats!B30</f>
         <v>38</v>
       </c>
-      <c r="D8" t="s">
-        <v>56</v>
-      </c>
-      <c r="E8" t="s">
+      <c r="D13" t="s">
+        <v>55</v>
+      </c>
+      <c r="E13" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>6</v>
+      </c>
+      <c r="B14" t="s">
+        <v>34</v>
+      </c>
+      <c r="C14">
+        <f>beats!B32</f>
+        <v>50</v>
+      </c>
+      <c r="D14" t="s">
+        <v>55</v>
+      </c>
+      <c r="E14" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>10</v>
+      </c>
+      <c r="B15" t="s">
+        <v>34</v>
+      </c>
+      <c r="C15">
+        <f>beats!B32</f>
+        <v>50</v>
+      </c>
+      <c r="D15" t="s">
+        <v>55</v>
+      </c>
+      <c r="E15" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>12</v>
+      </c>
+      <c r="B16" t="s">
+        <v>34</v>
+      </c>
+      <c r="C16">
+        <f>beats!B32</f>
+        <v>50</v>
+      </c>
+      <c r="D16" t="s">
+        <v>55</v>
+      </c>
+      <c r="E16" t="s">
         <v>136</v>
       </c>
     </row>

</xml_diff>

<commit_message>
corrected data to avoid spoilers
</commit_message>
<xml_diff>
--- a/TrailsTimeline.xlsx
+++ b/TrailsTimeline.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6da5a9201bc5826c/Documentos/trails_orbal_atlas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="201" documentId="13_ncr:1_{54315043-5A41-45C0-BA2E-F1BBE0C76030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8FA2D936-1E32-4BDA-A4CA-2992AFCAF86C}"/>
+  <xr:revisionPtr revIDLastSave="202" documentId="13_ncr:1_{54315043-5A41-45C0-BA2E-F1BBE0C76030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A916D030-FA83-449E-B860-C30A0DB664A9}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{B6393BEF-99C0-4DAE-AD63-40B518CD1F0D}"/>
   </bookViews>
@@ -471,9 +471,6 @@
     <t>Archeologist investigating the Tetracyclic towers</t>
   </si>
   <si>
-    <t>Disappeared on captured airliner</t>
-  </si>
-  <si>
     <t>Learning about Esmelas Crystal that needs retrieving from Mayor Klaus</t>
   </si>
   <si>
@@ -484,6 +481,9 @@
   </si>
   <si>
     <t>Widowed since the 100 day war</t>
+  </si>
+  <si>
+    <t>Disappeared on missing airliner</t>
   </si>
 </sst>
 </file>
@@ -542,6 +542,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1524,7 +1528,7 @@
         <v>35</v>
       </c>
       <c r="D13" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E13" t="s">
         <v>78</v>
@@ -2194,7 +2198,7 @@
         <v>55</v>
       </c>
       <c r="E2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -2212,7 +2216,7 @@
         <v>55</v>
       </c>
       <c r="E3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -2392,7 +2396,7 @@
         <v>55</v>
       </c>
       <c r="E13" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
@@ -2455,7 +2459,7 @@
         <v>55</v>
       </c>
       <c r="E16" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Updated faction display behavior
</commit_message>
<xml_diff>
--- a/TrailsTimeline.xlsx
+++ b/TrailsTimeline.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6da5a9201bc5826c/Documentos/trails_orbal_atlas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="202" documentId="13_ncr:1_{54315043-5A41-45C0-BA2E-F1BBE0C76030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A916D030-FA83-449E-B860-C30A0DB664A9}"/>
+  <xr:revisionPtr revIDLastSave="210" documentId="13_ncr:1_{54315043-5A41-45C0-BA2E-F1BBE0C76030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6C4B4E19-E496-44C0-9BB7-65FFA5F27261}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{B6393BEF-99C0-4DAE-AD63-40B518CD1F0D}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="380" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="149">
   <si>
     <t>char_id</t>
   </si>
@@ -484,6 +484,12 @@
   </si>
   <si>
     <t>Disappeared on missing airliner</t>
+  </si>
+  <si>
+    <t>former_faction</t>
+  </si>
+  <si>
+    <t>Jenis Royal Academy (cover identity)</t>
   </si>
 </sst>
 </file>
@@ -2145,12 +2151,12 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76C493BF-D343-46EF-AB39-E5F4461CCFFF}">
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="15.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15.85546875" customWidth="1"/>
-    <col min="4" max="4" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="70.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.28515625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="19.42578125" bestFit="1" customWidth="1"/>
@@ -2446,43 +2452,43 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>44</v>
+      </c>
+      <c r="B16" t="s">
+        <v>34</v>
+      </c>
+      <c r="C16">
+        <f>beats!B24</f>
+        <v>32</v>
+      </c>
+      <c r="D16" t="s">
+        <v>147</v>
+      </c>
+      <c r="E16" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>14</v>
       </c>
-      <c r="B16" t="s">
-        <v>34</v>
-      </c>
-      <c r="C16">
+      <c r="B17" t="s">
+        <v>34</v>
+      </c>
+      <c r="C17">
         <f>beats!B30</f>
         <v>38</v>
       </c>
-      <c r="D16" t="s">
-        <v>55</v>
-      </c>
-      <c r="E16" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>6</v>
-      </c>
-      <c r="B17" t="s">
-        <v>34</v>
-      </c>
-      <c r="C17">
-        <f>beats!B32</f>
-        <v>50</v>
-      </c>
       <c r="D17" t="s">
         <v>55</v>
       </c>
       <c r="E17" t="s">
-        <v>76</v>
+        <v>146</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B18" t="s">
         <v>34</v>
@@ -2500,7 +2506,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B19" t="s">
         <v>34</v>
@@ -2513,6 +2519,24 @@
         <v>55</v>
       </c>
       <c r="E19" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>12</v>
+      </c>
+      <c r="B20" t="s">
+        <v>34</v>
+      </c>
+      <c r="C20">
+        <f>beats!B32</f>
+        <v>50</v>
+      </c>
+      <c r="D20" t="s">
+        <v>55</v>
+      </c>
+      <c r="E20" t="s">
         <v>136</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added Chapter 1 and images
</commit_message>
<xml_diff>
--- a/TrailsTimeline.xlsx
+++ b/TrailsTimeline.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6da5a9201bc5826c/Documentos/trails_orbal_atlas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="210" documentId="13_ncr:1_{54315043-5A41-45C0-BA2E-F1BBE0C76030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6C4B4E19-E496-44C0-9BB7-65FFA5F27261}"/>
+  <xr:revisionPtr revIDLastSave="721" documentId="13_ncr:1_{54315043-5A41-45C0-BA2E-F1BBE0C76030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B5B080B5-1DAC-446A-B7D1-74EE945A40D8}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{B6393BEF-99C0-4DAE-AD63-40B518CD1F0D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B6393BEF-99C0-4DAE-AD63-40B518CD1F0D}"/>
   </bookViews>
   <sheets>
     <sheet name="characters" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="868" uniqueCount="291">
   <si>
     <t>char_id</t>
   </si>
@@ -490,6 +490,432 @@
   </si>
   <si>
     <t>Jenis Royal Academy (cover identity)</t>
+  </si>
+  <si>
+    <t>Tagging along Estelle and Joshua on their search for Cassius</t>
+  </si>
+  <si>
+    <t>Talking to Lugran on the Bracer Guild about the situation</t>
+  </si>
+  <si>
+    <t>morgan</t>
+  </si>
+  <si>
+    <t>General Morgan</t>
+  </si>
+  <si>
+    <t>Liberl Army</t>
+  </si>
+  <si>
+    <t>General of the Liberl army</t>
+  </si>
+  <si>
+    <t>Dislikes the guild, and is not sharing information about the disappeared airliner</t>
+  </si>
+  <si>
+    <t>Learned about General Morgan and his dislike for the guild</t>
+  </si>
+  <si>
+    <t>Learned how General Morgan is not sharing infformation with the guild, and limiting their movements in regards to the Linde disappearance investigation</t>
+  </si>
+  <si>
+    <t>Registering with the guild, going to Mayor Maybelle for a request</t>
+  </si>
+  <si>
+    <t>Learn about the Mayor's request for bracers to investigate the incident, receive letter of introduction that would allow them to speak with Morgan about the Linde</t>
+  </si>
+  <si>
+    <t>Going to haken Gate to speak with Morgan</t>
+  </si>
+  <si>
+    <t>haken</t>
+  </si>
+  <si>
+    <t>Haken Gate</t>
+  </si>
+  <si>
+    <t>nebel</t>
+  </si>
+  <si>
+    <t>Nebel Valley</t>
+  </si>
+  <si>
+    <t>ravennue</t>
+  </si>
+  <si>
+    <t>Ravennue Village</t>
+  </si>
+  <si>
+    <t>amberl</t>
+  </si>
+  <si>
+    <t>Amberl Tower</t>
+  </si>
+  <si>
+    <t>valleria_shore</t>
+  </si>
+  <si>
+    <t>Valleria Lakeshore</t>
+  </si>
+  <si>
+    <t>krone_pass</t>
+  </si>
+  <si>
+    <t>Krone Pass</t>
+  </si>
+  <si>
+    <t>Morgan discloses the details, learn the Linde disappeared returning to Rolent, theorize it was hijacked by the Imperial Army for ransom or the cargo</t>
+  </si>
+  <si>
+    <t>Learn the Capua Sky Bandits actually captured the Linde, and are demanding a ransom</t>
+  </si>
+  <si>
+    <t>Captured the Linde alongside the rest of the Sky Pirates</t>
+  </si>
+  <si>
+    <t>Accidentally reveal Bracer affiliation, get kicked out and Scherazard begind having an argument with Morgan about the military and the guild</t>
+  </si>
+  <si>
+    <t>Believes the military is incompetent in situations like the Linde disappearance</t>
+  </si>
+  <si>
+    <t>Believes the Guild is incomepetent in situations like the Linde disappearance</t>
+  </si>
+  <si>
+    <t>Encounter a traveler from the Erebonia Empire while waiting, who attempts to follow the party to their conversation with Morgan before being shooed out</t>
+  </si>
+  <si>
+    <t>Learn the traveler is called Olivier Lenheim, and agree to travel with him to Bose City</t>
+  </si>
+  <si>
+    <t>Interrupted by the Erebonian traveler, who starts playing the lute and singing to difuse the situation</t>
+  </si>
+  <si>
+    <t>olivier</t>
+  </si>
+  <si>
+    <t>Erebonian Traveller</t>
+  </si>
+  <si>
+    <t>Bard</t>
+  </si>
+  <si>
+    <t>Wandeing bard and musician from the Empire, impossible to have a normal conversation with</t>
+  </si>
+  <si>
+    <t>Olivier Lenheim</t>
+  </si>
+  <si>
+    <t>Removing Bracer badges to not trigger Morgan while waiting for him to arrive</t>
+  </si>
+  <si>
+    <t>Got shooed out from the meeting with Morgan he tried to sneak into</t>
+  </si>
+  <si>
+    <t>Left after Olivier difused his argument with Scherazard</t>
+  </si>
+  <si>
+    <t>Leaves to sightsee Bose</t>
+  </si>
+  <si>
+    <t>Reporting to the Mayor and the Guild what happend with Morgan</t>
+  </si>
+  <si>
+    <t>Encountered the reporters Nial and Dorothy, who give the party a tip on the Linde's disappearance in exchange for up to date information</t>
+  </si>
+  <si>
+    <t>Decide to do some side-quests before pursuing the tip</t>
+  </si>
+  <si>
+    <t>Encounter Alba at Amberl Tower and rescue him, after which he departs back to Bose</t>
+  </si>
+  <si>
+    <t>Going to Ravennue Village in pursue of the tip</t>
+  </si>
+  <si>
+    <t>agate</t>
+  </si>
+  <si>
+    <t>Agate Crosner</t>
+  </si>
+  <si>
+    <t>Was rescued by Estelle and Joshua in Amberl Tower, but decides to return to Bose alone</t>
+  </si>
+  <si>
+    <t>Encounter Agate heading out of Ravennue, but he quickly leaves on another job after a short talk</t>
+  </si>
+  <si>
+    <t>On a Bracer job</t>
+  </si>
+  <si>
+    <t>Talk to Ravennue's mayor, encounter a kid that claims to have seen something the night the Linde disappeared</t>
+  </si>
+  <si>
+    <t>Go to Ravennue's mine followin the kids' lead. Encounter it locked, returned to the city to get it unlocked</t>
+  </si>
+  <si>
+    <t>Inside the mine, encounter Josette's brother emptying the Linde, confronted him but he manages to flee</t>
+  </si>
+  <si>
+    <t>Decide to investigate the Linde and notice it is empty</t>
+  </si>
+  <si>
+    <t>Morgan arrives with the army and arrests the party despite their pleas thinking they were lying, sending them to Haken Gate</t>
+  </si>
+  <si>
+    <t>At the dungeon cell, encounter Olivier, who had also been arrested for drinking Bose's most expensive wine</t>
+  </si>
+  <si>
+    <t>Helping the party to redeem himself for drinking Bose's most expensive wine</t>
+  </si>
+  <si>
+    <t>Senior Bracer on a solo quest</t>
+  </si>
+  <si>
+    <t>Arrested for drinking Bose's most expensive wine</t>
+  </si>
+  <si>
+    <t>Mayor Maybelle comes and frees everyone, including Olivier on the condition he helps the the party solve the case</t>
+  </si>
+  <si>
+    <t>At the same time the Capua Sky Bandits atatck Bose and steals almost every valuable item from the citizens of bose</t>
+  </si>
+  <si>
+    <t>alan</t>
+  </si>
+  <si>
+    <t>Alan Richard</t>
+  </si>
+  <si>
+    <t>Going to Bose to see what happened</t>
+  </si>
+  <si>
+    <t>Encounter Alan Richard, who apologizes for the armies behavior and allows the party to interrogate the citizens after they are done</t>
+  </si>
+  <si>
+    <t>Head of the Liber Army Intelligence Division</t>
+  </si>
+  <si>
+    <t>Investigating the assault in Bose by the Capua Sky bandits</t>
+  </si>
+  <si>
+    <t>Raided Bose with the Sky Bandits and stole almost everyone's valueable possesions</t>
+  </si>
+  <si>
+    <t>Wait for the Capua Sky Bandits to come back, Scherazard knocks out Olivier so he isn't exposed to danger by drinking him under the table</t>
+  </si>
+  <si>
+    <t>Heavy drinker</t>
+  </si>
+  <si>
+    <t>fc_ch2</t>
+  </si>
+  <si>
+    <t>Got knocked out trying to outdrink Scherazard</t>
+  </si>
+  <si>
+    <t>Tried outdrinking Scherazard and got knocked out</t>
+  </si>
+  <si>
+    <t>loewe</t>
+  </si>
+  <si>
+    <t>THAT guy</t>
+  </si>
+  <si>
+    <t>Unknown</t>
+  </si>
+  <si>
+    <t>Listened in to the Sky Bandit's conversation, who mention their oldest sibling has been behaving weirdly after meatting THAT guy</t>
+  </si>
+  <si>
+    <t>THAT guy arrives, saying the ransom payment is underway, and that the queen will pay it herself</t>
+  </si>
+  <si>
+    <t>Kyle, Josettes's borther, revelas their airship is parked near the lakeshore, the only possible place being Amberl Tower</t>
+  </si>
+  <si>
+    <t>The party decide to go to Amberl Tower in search of their ship, only ot find it heavily guarded</t>
+  </si>
+  <si>
+    <t>Olivier interrupts while they are planning their assault, saying he will tag along regardless of the obstacles, and suggests sneaking into their ship, wich somehow works</t>
+  </si>
+  <si>
+    <t>Finding a man named Lloyd who witnessed the Capua Sky Bandits alongside Valleria Lakeshore, and that they are coming back tonight</t>
+  </si>
+  <si>
+    <t>Finding a way through the maze to rescue the hostages and defeat the Sky Bandits</t>
+  </si>
+  <si>
+    <t>Rescued the hostages, fighting the Sky Pirates after they state how they would have killed the hostages after receiving the ransom</t>
+  </si>
+  <si>
+    <t>Linde is rescued, but Cassius is nowhere to be found, the captain saying Cassis got off as soon as the linde took off</t>
+  </si>
+  <si>
+    <t>Alan and the intelligence Division appear as teh Capua Sky Bandits try to flee and arrests them</t>
+  </si>
+  <si>
+    <t>Returning to Bose to report findings, received second recommendation letter</t>
+  </si>
+  <si>
+    <t>Also received a parcel intended for Cassius, with a black myserious orbment from someone named "K", and that he should take it to "R" for analysis</t>
+  </si>
+  <si>
+    <t>ruan</t>
+  </si>
+  <si>
+    <t>Ruan</t>
+  </si>
+  <si>
+    <t>ruan_city</t>
+  </si>
+  <si>
+    <t>Ruan City</t>
+  </si>
+  <si>
+    <t>Deciding to go to Ruan to obtain the next recommendation letter from the guild</t>
+  </si>
+  <si>
+    <t>Part ways with Olivier and Scherazard who are going back to Rolent</t>
+  </si>
+  <si>
+    <t>After separating, Olivier is seen talking with someone about a mission on an orbment. Scherazard confronts him, and Olivier confesses he is involved with the Imperial Governmnet</t>
+  </si>
+  <si>
+    <t>Chapter 2</t>
+  </si>
+  <si>
+    <t>Preparing to head back to the Sky Bandit base</t>
+  </si>
+  <si>
+    <t>Found themselves in Nebel Valley after boarding the ship, which was the Capua Sky Pirates' hideout</t>
+  </si>
+  <si>
+    <t>Left after informing the Sky Bandits that the ransom payment is coming</t>
+  </si>
+  <si>
+    <t>Going to Rolent with Scherazard</t>
+  </si>
+  <si>
+    <t>Defeated the Capua Sky Pirates, after which, their leader, and brother of Josette, states he has no memories of what happened after meeting THAT guy</t>
+  </si>
+  <si>
+    <t>Taken away by the Intelligence Division</t>
+  </si>
+  <si>
+    <t>Arrested the Capua Sky Bandits</t>
+  </si>
+  <si>
+    <t>Assures the Capua Sky Bandits that the ransom payment is coming</t>
+  </si>
+  <si>
+    <t>Arrested the Capua Sky Bandits while they tried fleeing</t>
+  </si>
+  <si>
+    <t>Arrested by the Intelligence Division after attempting to flee from the Bracer Guild operation</t>
+  </si>
+  <si>
+    <t>Never boarded the Linde, and has not been spotted since</t>
+  </si>
+  <si>
+    <t>Received second recommendation letter</t>
+  </si>
+  <si>
+    <t>Going to Rolent with Olivier</t>
+  </si>
+  <si>
+    <t>Received a parcel from Cassius with a letter stating they will find him if they keep climbing the bracer ranks, and that he cannot return until the end of the queen's birthday ceremony</t>
+  </si>
+  <si>
+    <t>Left a letter for Estelle and Joshua explaining he cannot come back until the Queen's birthday cermony</t>
+  </si>
+  <si>
+    <t>Urges Estelle and joshua to keep climbing the Bracer ranks to fins him</t>
+  </si>
+  <si>
+    <t>Received a parcel with a strange orbment to be analysed by "R"</t>
+  </si>
+  <si>
+    <t>Decided to head to Ruan to continue climbing the Bracer ranks</t>
+  </si>
+  <si>
+    <t>Is involved with the Erebonian Empire government, and has been communicating with them secretely during a "misison"</t>
+  </si>
+  <si>
+    <t>Suspects of Olivier of being a spy for the Erebonian Empire</t>
+  </si>
+  <si>
+    <t>Setting out for Ruan</t>
+  </si>
+  <si>
+    <t>fc_ch3</t>
+  </si>
+  <si>
+    <t>Stopping at the Krone Pass Checkpoint for the night</t>
+  </si>
+  <si>
+    <t>manoria</t>
+  </si>
+  <si>
+    <t>Manoria</t>
+  </si>
+  <si>
+    <t>jenis</t>
+  </si>
+  <si>
+    <t>sapphirl</t>
+  </si>
+  <si>
+    <t>Sapphirl Tower</t>
+  </si>
+  <si>
+    <t>letten</t>
+  </si>
+  <si>
+    <t>Air Lettern</t>
+  </si>
+  <si>
+    <t>varenne</t>
+  </si>
+  <si>
+    <t>Varenne Lighthouse</t>
+  </si>
+  <si>
+    <t>mercia</t>
+  </si>
+  <si>
+    <t>Mercia Orphanage</t>
+  </si>
+  <si>
+    <t>loeweFullBody1.webp</t>
+  </si>
+  <si>
+    <t>loewe1.webp</t>
+  </si>
+  <si>
+    <t>morganFullBody1.webp</t>
+  </si>
+  <si>
+    <t>agateFullBody1.webp</t>
+  </si>
+  <si>
+    <t>morgan1.webp</t>
+  </si>
+  <si>
+    <t>olivier1.png</t>
+  </si>
+  <si>
+    <t>olivierFullBody1.png</t>
+  </si>
+  <si>
+    <t>agate1.png</t>
+  </si>
+  <si>
+    <t>alan1.png</t>
+  </si>
+  <si>
+    <t>alanFullBody1.png</t>
   </si>
 </sst>
 </file>
@@ -871,10 +1297,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16250901-8053-4627-8044-9432C6A9EB89}">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="20.85546875" bestFit="1" customWidth="1"/>
@@ -1043,6 +1469,121 @@
         <v>116</v>
       </c>
     </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>151</v>
+      </c>
+      <c r="B8" t="s">
+        <v>152</v>
+      </c>
+      <c r="C8" t="s">
+        <v>153</v>
+      </c>
+      <c r="D8" t="s">
+        <v>161</v>
+      </c>
+      <c r="E8" t="s">
+        <v>67</v>
+      </c>
+      <c r="F8" t="s">
+        <v>285</v>
+      </c>
+      <c r="G8" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>182</v>
+      </c>
+      <c r="B9" t="s">
+        <v>183</v>
+      </c>
+      <c r="C9" t="s">
+        <v>184</v>
+      </c>
+      <c r="D9" t="s">
+        <v>161</v>
+      </c>
+      <c r="E9" t="s">
+        <v>67</v>
+      </c>
+      <c r="F9" t="s">
+        <v>286</v>
+      </c>
+      <c r="G9" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>196</v>
+      </c>
+      <c r="B10" t="s">
+        <v>197</v>
+      </c>
+      <c r="C10" t="s">
+        <v>8</v>
+      </c>
+      <c r="D10" t="s">
+        <v>165</v>
+      </c>
+      <c r="E10" t="s">
+        <v>67</v>
+      </c>
+      <c r="F10" t="s">
+        <v>288</v>
+      </c>
+      <c r="G10" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>212</v>
+      </c>
+      <c r="B11" t="s">
+        <v>213</v>
+      </c>
+      <c r="C11" t="s">
+        <v>153</v>
+      </c>
+      <c r="D11" t="s">
+        <v>80</v>
+      </c>
+      <c r="E11" t="s">
+        <v>67</v>
+      </c>
+      <c r="F11" t="s">
+        <v>289</v>
+      </c>
+      <c r="G11" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>224</v>
+      </c>
+      <c r="B12" t="s">
+        <v>225</v>
+      </c>
+      <c r="C12" t="s">
+        <v>226</v>
+      </c>
+      <c r="D12" t="s">
+        <v>169</v>
+      </c>
+      <c r="E12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F12" t="s">
+        <v>282</v>
+      </c>
+      <c r="G12" t="s">
+        <v>281</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1050,11 +1591,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBE7F938-F724-45B1-B18D-82E13C0D228D}">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -1266,6 +1807,298 @@
       </c>
       <c r="F11">
         <v>66.599999999999994</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>161</v>
+      </c>
+      <c r="B12" t="s">
+        <v>162</v>
+      </c>
+      <c r="C12" t="s">
+        <v>54</v>
+      </c>
+      <c r="D12" t="s">
+        <v>40</v>
+      </c>
+      <c r="E12">
+        <v>25.9</v>
+      </c>
+      <c r="F12">
+        <v>63.1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>163</v>
+      </c>
+      <c r="B13" t="s">
+        <v>164</v>
+      </c>
+      <c r="C13" t="s">
+        <v>54</v>
+      </c>
+      <c r="D13" t="s">
+        <v>40</v>
+      </c>
+      <c r="E13">
+        <v>28.9</v>
+      </c>
+      <c r="F13">
+        <v>66.5</v>
+      </c>
+      <c r="G13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>165</v>
+      </c>
+      <c r="B14" t="s">
+        <v>166</v>
+      </c>
+      <c r="C14" t="s">
+        <v>54</v>
+      </c>
+      <c r="D14" t="s">
+        <v>40</v>
+      </c>
+      <c r="E14">
+        <v>24.3</v>
+      </c>
+      <c r="F14">
+        <v>65.2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>167</v>
+      </c>
+      <c r="B15" t="s">
+        <v>168</v>
+      </c>
+      <c r="C15" t="s">
+        <v>54</v>
+      </c>
+      <c r="D15" t="s">
+        <v>40</v>
+      </c>
+      <c r="E15">
+        <v>26.2</v>
+      </c>
+      <c r="F15">
+        <v>67.900000000000006</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>169</v>
+      </c>
+      <c r="B16" t="s">
+        <v>170</v>
+      </c>
+      <c r="C16" t="s">
+        <v>54</v>
+      </c>
+      <c r="D16" t="s">
+        <v>40</v>
+      </c>
+      <c r="E16">
+        <v>26.8</v>
+      </c>
+      <c r="F16">
+        <v>68.599999999999994</v>
+      </c>
+      <c r="G16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>171</v>
+      </c>
+      <c r="B17" t="s">
+        <v>172</v>
+      </c>
+      <c r="C17" t="s">
+        <v>54</v>
+      </c>
+      <c r="D17" t="s">
+        <v>40</v>
+      </c>
+      <c r="E17">
+        <v>21.8</v>
+      </c>
+      <c r="F17">
+        <v>67.599999999999994</v>
+      </c>
+      <c r="G17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>239</v>
+      </c>
+      <c r="B18" t="s">
+        <v>240</v>
+      </c>
+      <c r="C18" t="s">
+        <v>23</v>
+      </c>
+      <c r="D18" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>241</v>
+      </c>
+      <c r="B19" t="s">
+        <v>242</v>
+      </c>
+      <c r="C19" t="s">
+        <v>239</v>
+      </c>
+      <c r="D19" t="s">
+        <v>24</v>
+      </c>
+      <c r="E19">
+        <v>23.3</v>
+      </c>
+      <c r="F19">
+        <v>72.7</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>270</v>
+      </c>
+      <c r="B20" t="s">
+        <v>271</v>
+      </c>
+      <c r="C20" t="s">
+        <v>239</v>
+      </c>
+      <c r="D20" t="s">
+        <v>40</v>
+      </c>
+      <c r="E20">
+        <v>21.5</v>
+      </c>
+      <c r="F20">
+        <v>71.5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>272</v>
+      </c>
+      <c r="B21" t="s">
+        <v>46</v>
+      </c>
+      <c r="C21" t="s">
+        <v>239</v>
+      </c>
+      <c r="D21" t="s">
+        <v>40</v>
+      </c>
+      <c r="E21">
+        <v>25.1</v>
+      </c>
+      <c r="F21">
+        <v>70.599999999999994</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>273</v>
+      </c>
+      <c r="B22" t="s">
+        <v>274</v>
+      </c>
+      <c r="C22" t="s">
+        <v>239</v>
+      </c>
+      <c r="D22" t="s">
+        <v>40</v>
+      </c>
+      <c r="E22">
+        <v>23.6</v>
+      </c>
+      <c r="F22">
+        <v>74.099999999999994</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>275</v>
+      </c>
+      <c r="B23" t="s">
+        <v>276</v>
+      </c>
+      <c r="C23" t="s">
+        <v>239</v>
+      </c>
+      <c r="D23" t="s">
+        <v>40</v>
+      </c>
+      <c r="E23">
+        <v>24.3</v>
+      </c>
+      <c r="F23">
+        <v>75</v>
+      </c>
+      <c r="G23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>277</v>
+      </c>
+      <c r="B24" t="s">
+        <v>278</v>
+      </c>
+      <c r="C24" t="s">
+        <v>239</v>
+      </c>
+      <c r="D24" t="s">
+        <v>40</v>
+      </c>
+      <c r="E24">
+        <v>21.3</v>
+      </c>
+      <c r="F24">
+        <v>73.400000000000006</v>
+      </c>
+      <c r="G24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>279</v>
+      </c>
+      <c r="B25" t="s">
+        <v>280</v>
+      </c>
+      <c r="C25" t="s">
+        <v>239</v>
+      </c>
+      <c r="D25" t="s">
+        <v>40</v>
+      </c>
+      <c r="E25">
+        <v>21.9</v>
+      </c>
+      <c r="F25">
+        <v>70.400000000000006</v>
+      </c>
+      <c r="G25">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1275,10 +2108,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{94EA2C8E-D265-418D-8065-F972E277CAB9}">
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F82"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="78.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="162.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11.85546875" bestFit="1" customWidth="1"/>
   </cols>
@@ -1908,7 +2741,7 @@
         <v>67</v>
       </c>
       <c r="B32">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C32" t="s">
         <v>68</v>
@@ -1920,6 +2753,1006 @@
         <v>80</v>
       </c>
       <c r="F32" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>67</v>
+      </c>
+      <c r="B33">
+        <v>41</v>
+      </c>
+      <c r="C33" t="s">
+        <v>68</v>
+      </c>
+      <c r="D33" t="s">
+        <v>150</v>
+      </c>
+      <c r="E33" t="s">
+        <v>80</v>
+      </c>
+      <c r="F33" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>67</v>
+      </c>
+      <c r="B34">
+        <v>42</v>
+      </c>
+      <c r="C34" t="s">
+        <v>68</v>
+      </c>
+      <c r="D34" t="s">
+        <v>156</v>
+      </c>
+      <c r="E34" t="s">
+        <v>80</v>
+      </c>
+      <c r="F34" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>67</v>
+      </c>
+      <c r="B35">
+        <v>43</v>
+      </c>
+      <c r="C35" t="s">
+        <v>68</v>
+      </c>
+      <c r="D35" t="s">
+        <v>157</v>
+      </c>
+      <c r="E35" t="s">
+        <v>80</v>
+      </c>
+      <c r="F35" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>67</v>
+      </c>
+      <c r="B36">
+        <v>44</v>
+      </c>
+      <c r="C36" t="s">
+        <v>68</v>
+      </c>
+      <c r="D36" t="s">
+        <v>158</v>
+      </c>
+      <c r="E36" t="s">
+        <v>80</v>
+      </c>
+      <c r="F36" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>67</v>
+      </c>
+      <c r="B37">
+        <v>45</v>
+      </c>
+      <c r="C37" t="s">
+        <v>68</v>
+      </c>
+      <c r="D37" t="s">
+        <v>159</v>
+      </c>
+      <c r="E37" t="s">
+        <v>80</v>
+      </c>
+      <c r="F37" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>67</v>
+      </c>
+      <c r="B38">
+        <v>46</v>
+      </c>
+      <c r="C38" t="s">
+        <v>68</v>
+      </c>
+      <c r="D38" t="s">
+        <v>160</v>
+      </c>
+      <c r="E38" t="s">
+        <v>161</v>
+      </c>
+      <c r="F38" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>67</v>
+      </c>
+      <c r="B39">
+        <v>47</v>
+      </c>
+      <c r="C39" t="s">
+        <v>68</v>
+      </c>
+      <c r="D39" t="s">
+        <v>187</v>
+      </c>
+      <c r="E39" t="s">
+        <v>161</v>
+      </c>
+      <c r="F39" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>67</v>
+      </c>
+      <c r="B40">
+        <v>48</v>
+      </c>
+      <c r="C40" t="s">
+        <v>68</v>
+      </c>
+      <c r="D40" t="s">
+        <v>179</v>
+      </c>
+      <c r="E40" t="s">
+        <v>161</v>
+      </c>
+      <c r="F40" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>67</v>
+      </c>
+      <c r="B41">
+        <v>49</v>
+      </c>
+      <c r="C41" t="s">
+        <v>68</v>
+      </c>
+      <c r="D41" t="s">
+        <v>173</v>
+      </c>
+      <c r="E41" t="s">
+        <v>161</v>
+      </c>
+      <c r="F41" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>67</v>
+      </c>
+      <c r="B42">
+        <v>50</v>
+      </c>
+      <c r="C42" t="s">
+        <v>68</v>
+      </c>
+      <c r="D42" t="s">
+        <v>174</v>
+      </c>
+      <c r="E42" t="s">
+        <v>161</v>
+      </c>
+      <c r="F42" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>67</v>
+      </c>
+      <c r="B43">
+        <v>51</v>
+      </c>
+      <c r="C43" t="s">
+        <v>68</v>
+      </c>
+      <c r="D43" t="s">
+        <v>176</v>
+      </c>
+      <c r="E43" t="s">
+        <v>161</v>
+      </c>
+      <c r="F43" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>67</v>
+      </c>
+      <c r="B44">
+        <v>52</v>
+      </c>
+      <c r="C44" t="s">
+        <v>68</v>
+      </c>
+      <c r="D44" t="s">
+        <v>181</v>
+      </c>
+      <c r="E44" t="s">
+        <v>161</v>
+      </c>
+      <c r="F44" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>67</v>
+      </c>
+      <c r="B45">
+        <v>53</v>
+      </c>
+      <c r="C45" t="s">
+        <v>68</v>
+      </c>
+      <c r="D45" t="s">
+        <v>180</v>
+      </c>
+      <c r="E45" t="s">
+        <v>80</v>
+      </c>
+      <c r="F45" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>67</v>
+      </c>
+      <c r="B46">
+        <v>54</v>
+      </c>
+      <c r="C46" t="s">
+        <v>68</v>
+      </c>
+      <c r="D46" t="s">
+        <v>191</v>
+      </c>
+      <c r="E46" t="s">
+        <v>80</v>
+      </c>
+      <c r="F46" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>67</v>
+      </c>
+      <c r="B47">
+        <v>55</v>
+      </c>
+      <c r="C47" t="s">
+        <v>68</v>
+      </c>
+      <c r="D47" t="s">
+        <v>192</v>
+      </c>
+      <c r="E47" t="s">
+        <v>80</v>
+      </c>
+      <c r="F47" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>67</v>
+      </c>
+      <c r="B48">
+        <v>56</v>
+      </c>
+      <c r="C48" t="s">
+        <v>68</v>
+      </c>
+      <c r="D48" t="s">
+        <v>193</v>
+      </c>
+      <c r="E48" t="s">
+        <v>80</v>
+      </c>
+      <c r="F48" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>67</v>
+      </c>
+      <c r="B49">
+        <v>57</v>
+      </c>
+      <c r="C49" t="s">
+        <v>68</v>
+      </c>
+      <c r="D49" t="s">
+        <v>194</v>
+      </c>
+      <c r="E49" t="s">
+        <v>167</v>
+      </c>
+      <c r="F49" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>67</v>
+      </c>
+      <c r="B50">
+        <v>58</v>
+      </c>
+      <c r="C50" t="s">
+        <v>68</v>
+      </c>
+      <c r="D50" t="s">
+        <v>195</v>
+      </c>
+      <c r="E50" t="s">
+        <v>165</v>
+      </c>
+      <c r="F50" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>67</v>
+      </c>
+      <c r="B51">
+        <v>59</v>
+      </c>
+      <c r="C51" t="s">
+        <v>68</v>
+      </c>
+      <c r="D51" t="s">
+        <v>199</v>
+      </c>
+      <c r="E51" t="s">
+        <v>165</v>
+      </c>
+      <c r="F51" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>67</v>
+      </c>
+      <c r="B52">
+        <v>60</v>
+      </c>
+      <c r="C52" t="s">
+        <v>68</v>
+      </c>
+      <c r="D52" t="s">
+        <v>201</v>
+      </c>
+      <c r="E52" t="s">
+        <v>165</v>
+      </c>
+      <c r="F52" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>67</v>
+      </c>
+      <c r="B53">
+        <v>61</v>
+      </c>
+      <c r="C53" t="s">
+        <v>68</v>
+      </c>
+      <c r="D53" t="s">
+        <v>202</v>
+      </c>
+      <c r="E53" t="s">
+        <v>165</v>
+      </c>
+      <c r="F53" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>67</v>
+      </c>
+      <c r="B54">
+        <v>62</v>
+      </c>
+      <c r="C54" t="s">
+        <v>68</v>
+      </c>
+      <c r="D54" t="s">
+        <v>203</v>
+      </c>
+      <c r="E54" t="s">
+        <v>165</v>
+      </c>
+      <c r="F54" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>67</v>
+      </c>
+      <c r="B55">
+        <v>63</v>
+      </c>
+      <c r="C55" t="s">
+        <v>68</v>
+      </c>
+      <c r="D55" t="s">
+        <v>204</v>
+      </c>
+      <c r="E55" t="s">
+        <v>165</v>
+      </c>
+      <c r="F55" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>67</v>
+      </c>
+      <c r="B56">
+        <v>64</v>
+      </c>
+      <c r="C56" t="s">
+        <v>68</v>
+      </c>
+      <c r="D56" t="s">
+        <v>205</v>
+      </c>
+      <c r="E56" t="s">
+        <v>165</v>
+      </c>
+      <c r="F56" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>67</v>
+      </c>
+      <c r="B57">
+        <v>65</v>
+      </c>
+      <c r="C57" t="s">
+        <v>68</v>
+      </c>
+      <c r="D57" t="s">
+        <v>206</v>
+      </c>
+      <c r="E57" t="s">
+        <v>161</v>
+      </c>
+      <c r="F57" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>67</v>
+      </c>
+      <c r="B58">
+        <v>66</v>
+      </c>
+      <c r="C58" t="s">
+        <v>68</v>
+      </c>
+      <c r="D58" t="s">
+        <v>210</v>
+      </c>
+      <c r="E58" t="s">
+        <v>161</v>
+      </c>
+      <c r="F58" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>67</v>
+      </c>
+      <c r="B59">
+        <v>67</v>
+      </c>
+      <c r="C59" t="s">
+        <v>68</v>
+      </c>
+      <c r="D59" t="s">
+        <v>211</v>
+      </c>
+      <c r="E59" t="s">
+        <v>80</v>
+      </c>
+      <c r="F59" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>67</v>
+      </c>
+      <c r="B60">
+        <v>68</v>
+      </c>
+      <c r="C60" t="s">
+        <v>68</v>
+      </c>
+      <c r="D60" t="s">
+        <v>214</v>
+      </c>
+      <c r="E60" t="s">
+        <v>80</v>
+      </c>
+      <c r="F60" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>67</v>
+      </c>
+      <c r="B61">
+        <v>69</v>
+      </c>
+      <c r="C61" t="s">
+        <v>68</v>
+      </c>
+      <c r="D61" t="s">
+        <v>215</v>
+      </c>
+      <c r="E61" t="s">
+        <v>80</v>
+      </c>
+      <c r="F61" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>67</v>
+      </c>
+      <c r="B62">
+        <v>70</v>
+      </c>
+      <c r="C62" t="s">
+        <v>68</v>
+      </c>
+      <c r="D62" t="s">
+        <v>232</v>
+      </c>
+      <c r="E62" t="s">
+        <v>80</v>
+      </c>
+      <c r="F62" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>67</v>
+      </c>
+      <c r="B63">
+        <v>71</v>
+      </c>
+      <c r="C63" t="s">
+        <v>68</v>
+      </c>
+      <c r="D63" t="s">
+        <v>219</v>
+      </c>
+      <c r="E63" t="s">
+        <v>169</v>
+      </c>
+      <c r="F63" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>67</v>
+      </c>
+      <c r="B64">
+        <v>72</v>
+      </c>
+      <c r="C64" t="s">
+        <v>68</v>
+      </c>
+      <c r="D64" t="s">
+        <v>227</v>
+      </c>
+      <c r="E64" t="s">
+        <v>169</v>
+      </c>
+      <c r="F64" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>67</v>
+      </c>
+      <c r="B65">
+        <v>73</v>
+      </c>
+      <c r="C65" t="s">
+        <v>68</v>
+      </c>
+      <c r="D65" t="s">
+        <v>228</v>
+      </c>
+      <c r="E65" t="s">
+        <v>169</v>
+      </c>
+      <c r="F65" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>67</v>
+      </c>
+      <c r="B66">
+        <v>74</v>
+      </c>
+      <c r="C66" t="s">
+        <v>68</v>
+      </c>
+      <c r="D66" t="s">
+        <v>229</v>
+      </c>
+      <c r="E66" t="s">
+        <v>169</v>
+      </c>
+      <c r="F66" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>67</v>
+      </c>
+      <c r="B67">
+        <v>75</v>
+      </c>
+      <c r="C67" t="s">
+        <v>68</v>
+      </c>
+      <c r="D67" t="s">
+        <v>230</v>
+      </c>
+      <c r="E67" t="s">
+        <v>167</v>
+      </c>
+      <c r="F67" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>67</v>
+      </c>
+      <c r="B68">
+        <v>76</v>
+      </c>
+      <c r="C68" t="s">
+        <v>68</v>
+      </c>
+      <c r="D68" t="s">
+        <v>231</v>
+      </c>
+      <c r="E68" t="s">
+        <v>167</v>
+      </c>
+      <c r="F68" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>67</v>
+      </c>
+      <c r="B69">
+        <v>77</v>
+      </c>
+      <c r="C69" t="s">
+        <v>68</v>
+      </c>
+      <c r="D69" t="s">
+        <v>248</v>
+      </c>
+      <c r="E69" t="s">
+        <v>163</v>
+      </c>
+      <c r="F69" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>67</v>
+      </c>
+      <c r="B70">
+        <v>78</v>
+      </c>
+      <c r="C70" t="s">
+        <v>68</v>
+      </c>
+      <c r="D70" t="s">
+        <v>233</v>
+      </c>
+      <c r="E70" t="s">
+        <v>163</v>
+      </c>
+      <c r="F70" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>67</v>
+      </c>
+      <c r="B71">
+        <v>79</v>
+      </c>
+      <c r="C71" t="s">
+        <v>68</v>
+      </c>
+      <c r="D71" t="s">
+        <v>234</v>
+      </c>
+      <c r="E71" t="s">
+        <v>163</v>
+      </c>
+      <c r="F71" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>67</v>
+      </c>
+      <c r="B72">
+        <v>80</v>
+      </c>
+      <c r="C72" t="s">
+        <v>68</v>
+      </c>
+      <c r="D72" t="s">
+        <v>251</v>
+      </c>
+      <c r="E72" t="s">
+        <v>163</v>
+      </c>
+      <c r="F72" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>67</v>
+      </c>
+      <c r="B73">
+        <v>81</v>
+      </c>
+      <c r="C73" t="s">
+        <v>68</v>
+      </c>
+      <c r="D73" t="s">
+        <v>236</v>
+      </c>
+      <c r="E73" t="s">
+        <v>163</v>
+      </c>
+      <c r="F73" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>67</v>
+      </c>
+      <c r="B74">
+        <v>82</v>
+      </c>
+      <c r="C74" t="s">
+        <v>68</v>
+      </c>
+      <c r="D74" t="s">
+        <v>235</v>
+      </c>
+      <c r="E74" t="s">
+        <v>163</v>
+      </c>
+      <c r="F74" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>67</v>
+      </c>
+      <c r="B75">
+        <v>83</v>
+      </c>
+      <c r="C75" t="s">
+        <v>68</v>
+      </c>
+      <c r="D75" t="s">
+        <v>237</v>
+      </c>
+      <c r="E75" t="s">
+        <v>80</v>
+      </c>
+      <c r="F75" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>67</v>
+      </c>
+      <c r="B76">
+        <v>84</v>
+      </c>
+      <c r="C76" t="s">
+        <v>68</v>
+      </c>
+      <c r="D76" t="s">
+        <v>260</v>
+      </c>
+      <c r="E76" t="s">
+        <v>80</v>
+      </c>
+      <c r="F76" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>67</v>
+      </c>
+      <c r="B77">
+        <v>85</v>
+      </c>
+      <c r="C77" t="s">
+        <v>68</v>
+      </c>
+      <c r="D77" t="s">
+        <v>238</v>
+      </c>
+      <c r="E77" t="s">
+        <v>80</v>
+      </c>
+      <c r="F77" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>67</v>
+      </c>
+      <c r="B78">
+        <v>86</v>
+      </c>
+      <c r="C78" t="s">
+        <v>68</v>
+      </c>
+      <c r="D78" t="s">
+        <v>243</v>
+      </c>
+      <c r="E78" t="s">
+        <v>80</v>
+      </c>
+      <c r="F78" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>67</v>
+      </c>
+      <c r="B79">
+        <v>87</v>
+      </c>
+      <c r="C79" t="s">
+        <v>68</v>
+      </c>
+      <c r="D79" t="s">
+        <v>244</v>
+      </c>
+      <c r="E79" t="s">
+        <v>80</v>
+      </c>
+      <c r="F79" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>67</v>
+      </c>
+      <c r="B80">
+        <v>88</v>
+      </c>
+      <c r="C80" t="s">
+        <v>68</v>
+      </c>
+      <c r="D80" t="s">
+        <v>245</v>
+      </c>
+      <c r="E80" t="s">
+        <v>80</v>
+      </c>
+      <c r="F80" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>221</v>
+      </c>
+      <c r="B81">
+        <v>89</v>
+      </c>
+      <c r="C81" t="s">
+        <v>246</v>
+      </c>
+      <c r="D81" t="s">
+        <v>267</v>
+      </c>
+      <c r="E81" t="s">
+        <v>80</v>
+      </c>
+      <c r="F81" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>268</v>
+      </c>
+      <c r="B82">
+        <v>90</v>
+      </c>
+      <c r="C82" t="s">
+        <v>246</v>
+      </c>
+      <c r="D82" t="s">
+        <v>269</v>
+      </c>
+      <c r="E82" t="s">
+        <v>171</v>
+      </c>
+      <c r="F82" t="s">
         <v>69</v>
       </c>
     </row>
@@ -1931,14 +3764,14 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83D801B6-5B2D-4C63-87A9-B0F352D632BD}">
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10.28515625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="40.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="76.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -2115,6 +3948,12 @@
         <f>beats!B22</f>
         <v>30</v>
       </c>
+      <c r="E9" t="s">
+        <v>67</v>
+      </c>
+      <c r="F9">
+        <v>50</v>
+      </c>
       <c r="G9" t="s">
         <v>110</v>
       </c>
@@ -2144,21 +3983,361 @@
         <v>65</v>
       </c>
     </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" t="s">
+        <v>67</v>
+      </c>
+      <c r="C11">
+        <f>beats!B32</f>
+        <v>40</v>
+      </c>
+      <c r="E11" t="s">
+        <v>67</v>
+      </c>
+      <c r="F11">
+        <f>beats!B80</f>
+        <v>88</v>
+      </c>
+      <c r="G11" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>182</v>
+      </c>
+      <c r="B12" t="s">
+        <v>67</v>
+      </c>
+      <c r="C12">
+        <f>beats!B40</f>
+        <v>48</v>
+      </c>
+      <c r="E12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F12">
+        <f>beats!B41</f>
+        <v>49</v>
+      </c>
+      <c r="G12" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>151</v>
+      </c>
+      <c r="B13" t="s">
+        <v>67</v>
+      </c>
+      <c r="C13">
+        <f>beats!B40</f>
+        <v>48</v>
+      </c>
+      <c r="E13" t="s">
+        <v>67</v>
+      </c>
+      <c r="F13">
+        <f>beats!B44</f>
+        <v>52</v>
+      </c>
+      <c r="G13" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>182</v>
+      </c>
+      <c r="B14" t="s">
+        <v>67</v>
+      </c>
+      <c r="C14">
+        <f>beats!B44</f>
+        <v>52</v>
+      </c>
+      <c r="E14" t="s">
+        <v>67</v>
+      </c>
+      <c r="F14">
+        <f>beats!B46</f>
+        <v>54</v>
+      </c>
+      <c r="G14" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>196</v>
+      </c>
+      <c r="B15" t="s">
+        <v>67</v>
+      </c>
+      <c r="C15">
+        <f>beats!B51</f>
+        <v>59</v>
+      </c>
+      <c r="E15" t="s">
+        <v>67</v>
+      </c>
+      <c r="F15">
+        <f>beats!B51</f>
+        <v>59</v>
+      </c>
+      <c r="G15" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>182</v>
+      </c>
+      <c r="B16" t="s">
+        <v>67</v>
+      </c>
+      <c r="C16">
+        <f>beats!B57</f>
+        <v>65</v>
+      </c>
+      <c r="E16" t="s">
+        <v>67</v>
+      </c>
+      <c r="F16">
+        <f>beats!B63</f>
+        <v>71</v>
+      </c>
+      <c r="G16" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>44</v>
+      </c>
+      <c r="B17" t="s">
+        <v>67</v>
+      </c>
+      <c r="C17">
+        <f>beats!B59</f>
+        <v>67</v>
+      </c>
+      <c r="D17" t="s">
+        <v>80</v>
+      </c>
+      <c r="E17" t="s">
+        <v>67</v>
+      </c>
+      <c r="F17">
+        <f>beats!B59</f>
+        <v>67</v>
+      </c>
+      <c r="G17" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>212</v>
+      </c>
+      <c r="B18" t="s">
+        <v>67</v>
+      </c>
+      <c r="C18">
+        <f>beats!B61</f>
+        <v>69</v>
+      </c>
+      <c r="E18" t="s">
+        <v>67</v>
+      </c>
+      <c r="F18">
+        <f>beats!B61</f>
+        <v>69</v>
+      </c>
+      <c r="G18" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>182</v>
+      </c>
+      <c r="B19" t="s">
+        <v>67</v>
+      </c>
+      <c r="C19">
+        <f>beats!B63</f>
+        <v>71</v>
+      </c>
+      <c r="E19" t="s">
+        <v>67</v>
+      </c>
+      <c r="F19">
+        <f>beats!B63</f>
+        <v>71</v>
+      </c>
+      <c r="G19" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>44</v>
+      </c>
+      <c r="B20" t="s">
+        <v>67</v>
+      </c>
+      <c r="C20">
+        <f>beats!B64</f>
+        <v>72</v>
+      </c>
+      <c r="E20" t="s">
+        <v>67</v>
+      </c>
+      <c r="F20">
+        <f>beats!B66</f>
+        <v>74</v>
+      </c>
+      <c r="G20" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>224</v>
+      </c>
+      <c r="B21" t="s">
+        <v>67</v>
+      </c>
+      <c r="C21">
+        <f>beats!B65</f>
+        <v>73</v>
+      </c>
+      <c r="E21" t="s">
+        <v>67</v>
+      </c>
+      <c r="F21">
+        <f>beats!B66</f>
+        <v>74</v>
+      </c>
+      <c r="G21" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>182</v>
+      </c>
+      <c r="B22" t="s">
+        <v>67</v>
+      </c>
+      <c r="C22">
+        <f>beats!B68</f>
+        <v>76</v>
+      </c>
+      <c r="D22" t="s">
+        <v>78</v>
+      </c>
+      <c r="E22" t="s">
+        <v>67</v>
+      </c>
+      <c r="F22">
+        <f>beats!B80</f>
+        <v>88</v>
+      </c>
+      <c r="G22" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>44</v>
+      </c>
+      <c r="B23" t="s">
+        <v>67</v>
+      </c>
+      <c r="C23">
+        <f>beats!B71</f>
+        <v>79</v>
+      </c>
+      <c r="E23" t="s">
+        <v>67</v>
+      </c>
+      <c r="F23">
+        <f>beats!B73</f>
+        <v>81</v>
+      </c>
+      <c r="G23" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>212</v>
+      </c>
+      <c r="B24" t="s">
+        <v>67</v>
+      </c>
+      <c r="C24">
+        <f>beats!B73</f>
+        <v>81</v>
+      </c>
+      <c r="E24" t="s">
+        <v>67</v>
+      </c>
+      <c r="F24">
+        <f>beats!B73</f>
+        <v>81</v>
+      </c>
+      <c r="G24" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>12</v>
+      </c>
+      <c r="B25" t="s">
+        <v>67</v>
+      </c>
+      <c r="C25">
+        <f>beats!B80</f>
+        <v>88</v>
+      </c>
+      <c r="D25" t="s">
+        <v>78</v>
+      </c>
+      <c r="E25" t="s">
+        <v>67</v>
+      </c>
+      <c r="F25">
+        <f>beats!B80</f>
+        <v>88</v>
+      </c>
+      <c r="G25" t="s">
+        <v>259</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76C493BF-D343-46EF-AB39-E5F4461CCFFF}">
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H45"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="15.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15.85546875" customWidth="1"/>
     <col min="4" max="4" width="14" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="70.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="108.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.7109375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="19.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="20.28515625" bestFit="1" customWidth="1"/>
   </cols>
@@ -2468,7 +4647,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>14</v>
       </c>
@@ -2486,7 +4665,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>6</v>
       </c>
@@ -2495,7 +4674,7 @@
       </c>
       <c r="C18">
         <f>beats!B32</f>
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="D18" t="s">
         <v>55</v>
@@ -2504,7 +4683,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>10</v>
       </c>
@@ -2513,7 +4692,7 @@
       </c>
       <c r="C19">
         <f>beats!B32</f>
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="D19" t="s">
         <v>55</v>
@@ -2522,7 +4701,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>12</v>
       </c>
@@ -2531,13 +4710,400 @@
       </c>
       <c r="C20">
         <f>beats!B32</f>
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="D20" t="s">
         <v>55</v>
       </c>
       <c r="E20" t="s">
         <v>136</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>151</v>
+      </c>
+      <c r="B21" t="s">
+        <v>67</v>
+      </c>
+      <c r="C21">
+        <f>beats!B33</f>
+        <v>41</v>
+      </c>
+      <c r="D21" t="s">
+        <v>55</v>
+      </c>
+      <c r="E21" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>151</v>
+      </c>
+      <c r="B22" t="s">
+        <v>67</v>
+      </c>
+      <c r="C22">
+        <f>beats!B35</f>
+        <v>43</v>
+      </c>
+      <c r="D22" t="s">
+        <v>55</v>
+      </c>
+      <c r="E22" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>44</v>
+      </c>
+      <c r="B23" t="s">
+        <v>67</v>
+      </c>
+      <c r="C23">
+        <f>beats!B42</f>
+        <v>50</v>
+      </c>
+      <c r="D23" t="s">
+        <v>55</v>
+      </c>
+      <c r="E23" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>12</v>
+      </c>
+      <c r="C24">
+        <f>beats!B43</f>
+        <v>51</v>
+      </c>
+      <c r="D24" t="s">
+        <v>55</v>
+      </c>
+      <c r="E24" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>151</v>
+      </c>
+      <c r="C25">
+        <f>beats!B43</f>
+        <v>51</v>
+      </c>
+      <c r="D25" t="s">
+        <v>55</v>
+      </c>
+      <c r="E25" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>182</v>
+      </c>
+      <c r="C26">
+        <f>beats!B45</f>
+        <v>53</v>
+      </c>
+      <c r="D26" t="s">
+        <v>55</v>
+      </c>
+      <c r="E26" t="s">
+        <v>185</v>
+      </c>
+      <c r="F26" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>92</v>
+      </c>
+      <c r="C27">
+        <f>beats!B49</f>
+        <v>57</v>
+      </c>
+      <c r="D27" t="s">
+        <v>55</v>
+      </c>
+      <c r="E27" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>196</v>
+      </c>
+      <c r="C28">
+        <f>beats!B51</f>
+        <v>59</v>
+      </c>
+      <c r="D28" t="s">
+        <v>55</v>
+      </c>
+      <c r="E28" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>182</v>
+      </c>
+      <c r="C29">
+        <f>beats!B58</f>
+        <v>66</v>
+      </c>
+      <c r="D29" t="s">
+        <v>55</v>
+      </c>
+      <c r="E29" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>212</v>
+      </c>
+      <c r="C30">
+        <f>beats!B61</f>
+        <v>69</v>
+      </c>
+      <c r="D30" t="s">
+        <v>55</v>
+      </c>
+      <c r="E30" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>12</v>
+      </c>
+      <c r="C31">
+        <f>beats!B63</f>
+        <v>71</v>
+      </c>
+      <c r="D31" t="s">
+        <v>55</v>
+      </c>
+      <c r="E31" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>182</v>
+      </c>
+      <c r="C32">
+        <f>beats!B63</f>
+        <v>71</v>
+      </c>
+      <c r="D32" t="s">
+        <v>55</v>
+      </c>
+      <c r="E32" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>224</v>
+      </c>
+      <c r="C33">
+        <f>beats!B65</f>
+        <v>73</v>
+      </c>
+      <c r="D33" t="s">
+        <v>55</v>
+      </c>
+      <c r="E33" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>212</v>
+      </c>
+      <c r="C34">
+        <f>beats!B73</f>
+        <v>81</v>
+      </c>
+      <c r="D34" t="s">
+        <v>55</v>
+      </c>
+      <c r="E34" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>44</v>
+      </c>
+      <c r="C35">
+        <f>beats!B73</f>
+        <v>81</v>
+      </c>
+      <c r="D35" t="s">
+        <v>55</v>
+      </c>
+      <c r="E35" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>14</v>
+      </c>
+      <c r="C36">
+        <f>beats!B74</f>
+        <v>82</v>
+      </c>
+      <c r="D36" t="s">
+        <v>55</v>
+      </c>
+      <c r="E36" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>6</v>
+      </c>
+      <c r="C37">
+        <f>beats!B75</f>
+        <v>83</v>
+      </c>
+      <c r="D37" t="s">
+        <v>55</v>
+      </c>
+      <c r="E37" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>10</v>
+      </c>
+      <c r="C38">
+        <f>beats!B75</f>
+        <v>83</v>
+      </c>
+      <c r="D38" t="s">
+        <v>55</v>
+      </c>
+      <c r="E38" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>14</v>
+      </c>
+      <c r="C39">
+        <f>beats!B76</f>
+        <v>84</v>
+      </c>
+      <c r="D39" t="s">
+        <v>55</v>
+      </c>
+      <c r="E39" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>14</v>
+      </c>
+      <c r="C40">
+        <f>beats!B76</f>
+        <v>84</v>
+      </c>
+      <c r="D40" t="s">
+        <v>55</v>
+      </c>
+      <c r="E40" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>14</v>
+      </c>
+      <c r="C41">
+        <f>beats!B77</f>
+        <v>85</v>
+      </c>
+      <c r="D41" t="s">
+        <v>55</v>
+      </c>
+      <c r="E41" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>6</v>
+      </c>
+      <c r="C42">
+        <f>beats!B78</f>
+        <v>86</v>
+      </c>
+      <c r="D42" t="s">
+        <v>55</v>
+      </c>
+      <c r="E42" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>10</v>
+      </c>
+      <c r="C43">
+        <f>beats!B78</f>
+        <v>86</v>
+      </c>
+      <c r="D43" t="s">
+        <v>55</v>
+      </c>
+      <c r="E43" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>182</v>
+      </c>
+      <c r="C44">
+        <f>beats!B80</f>
+        <v>88</v>
+      </c>
+      <c r="D44" t="s">
+        <v>55</v>
+      </c>
+      <c r="E44" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>12</v>
+      </c>
+      <c r="C45">
+        <f>beats!B80</f>
+        <v>88</v>
+      </c>
+      <c r="D45" t="s">
+        <v>55</v>
+      </c>
+      <c r="E45" t="s">
+        <v>266</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added routes, corrected data
</commit_message>
<xml_diff>
--- a/TrailsTimeline.xlsx
+++ b/TrailsTimeline.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6da5a9201bc5826c/Documentos/trails_orbal_atlas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="721" documentId="13_ncr:1_{54315043-5A41-45C0-BA2E-F1BBE0C76030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B5B080B5-1DAC-446A-B7D1-74EE945A40D8}"/>
+  <xr:revisionPtr revIDLastSave="734" documentId="13_ncr:1_{54315043-5A41-45C0-BA2E-F1BBE0C76030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{03FB0DDA-9D43-4941-A99F-19FFE3DDFF16}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B6393BEF-99C0-4DAE-AD63-40B518CD1F0D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{B6393BEF-99C0-4DAE-AD63-40B518CD1F0D}"/>
   </bookViews>
   <sheets>
     <sheet name="characters" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="868" uniqueCount="291">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="872" uniqueCount="292">
   <si>
     <t>char_id</t>
   </si>
@@ -916,6 +916,9 @@
   </si>
   <si>
     <t>alanFullBody1.png</t>
+  </si>
+  <si>
+    <t>Accompanying the gang to the Sky Bandit hideout</t>
   </si>
 </sst>
 </file>
@@ -3764,7 +3767,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83D801B6-5B2D-4C63-87A9-B0F352D632BD}">
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="13.85546875" bestFit="1" customWidth="1"/>
@@ -4239,9 +4242,6 @@
         <f>beats!B68</f>
         <v>76</v>
       </c>
-      <c r="D22" t="s">
-        <v>78</v>
-      </c>
       <c r="E22" t="s">
         <v>67</v>
       </c>
@@ -4250,7 +4250,7 @@
         <v>88</v>
       </c>
       <c r="G22" t="s">
-        <v>250</v>
+        <v>291</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
@@ -4320,6 +4320,31 @@
       </c>
       <c r="G25" t="s">
         <v>259</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>182</v>
+      </c>
+      <c r="B26" t="s">
+        <v>67</v>
+      </c>
+      <c r="C26">
+        <f>beats!B80</f>
+        <v>88</v>
+      </c>
+      <c r="D26" t="s">
+        <v>78</v>
+      </c>
+      <c r="E26" t="s">
+        <v>67</v>
+      </c>
+      <c r="F26">
+        <f>beats!B80</f>
+        <v>88</v>
+      </c>
+      <c r="G26" t="s">
+        <v>250</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated route behavior and some visual effects
</commit_message>
<xml_diff>
--- a/TrailsTimeline.xlsx
+++ b/TrailsTimeline.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6da5a9201bc5826c/Documentos/trails_orbal_atlas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="734" documentId="13_ncr:1_{54315043-5A41-45C0-BA2E-F1BBE0C76030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{03FB0DDA-9D43-4941-A99F-19FFE3DDFF16}"/>
+  <xr:revisionPtr revIDLastSave="765" documentId="13_ncr:1_{54315043-5A41-45C0-BA2E-F1BBE0C76030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A309053C-3586-48E4-AA7D-596D7AEC7E8E}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{B6393BEF-99C0-4DAE-AD63-40B518CD1F0D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{B6393BEF-99C0-4DAE-AD63-40B518CD1F0D}"/>
   </bookViews>
   <sheets>
     <sheet name="characters" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="872" uniqueCount="292">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="911" uniqueCount="297">
   <si>
     <t>char_id</t>
   </si>
@@ -919,6 +919,21 @@
   </si>
   <si>
     <t>Accompanying the gang to the Sky Bandit hideout</t>
+  </si>
+  <si>
+    <t>Arrested the Bracers beleiving they kidnapped the Linde</t>
+  </si>
+  <si>
+    <t>Josette's brother started acting weird after meeting him</t>
+  </si>
+  <si>
+    <t>Suspicious of THAT guy as his brother started acting weird after meeting him</t>
+  </si>
+  <si>
+    <t>travel_mode</t>
+  </si>
+  <si>
+    <t>air</t>
   </si>
 </sst>
 </file>
@@ -2111,15 +2126,16 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{94EA2C8E-D265-418D-8065-F972E277CAB9}">
-  <dimension ref="A1:F82"/>
+  <dimension ref="A1:G82"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="162.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>27</v>
       </c>
@@ -2138,8 +2154,11 @@
       <c r="F1" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>34</v>
       </c>
@@ -2159,7 +2178,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>34</v>
       </c>
@@ -2179,7 +2198,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>34</v>
       </c>
@@ -2199,7 +2218,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>34</v>
       </c>
@@ -2219,7 +2238,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>34</v>
       </c>
@@ -2239,7 +2258,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>34</v>
       </c>
@@ -2259,7 +2278,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>34</v>
       </c>
@@ -2279,7 +2298,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>34</v>
       </c>
@@ -2299,7 +2318,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>34</v>
       </c>
@@ -2319,7 +2338,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>34</v>
       </c>
@@ -2339,7 +2358,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>34</v>
       </c>
@@ -2359,7 +2378,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>34</v>
       </c>
@@ -2379,7 +2398,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>34</v>
       </c>
@@ -2399,7 +2418,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>34</v>
       </c>
@@ -2419,7 +2438,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>34</v>
       </c>
@@ -3293,7 +3312,7 @@
         <v>211</v>
       </c>
       <c r="E59" t="s">
-        <v>80</v>
+        <v>161</v>
       </c>
       <c r="F59" t="s">
         <v>69</v>
@@ -3399,7 +3418,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>67</v>
       </c>
@@ -3419,7 +3438,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>67</v>
       </c>
@@ -3439,7 +3458,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>67</v>
       </c>
@@ -3459,7 +3478,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>67</v>
       </c>
@@ -3479,7 +3498,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>67</v>
       </c>
@@ -3498,8 +3517,11 @@
       <c r="F69" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G69" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>67</v>
       </c>
@@ -3519,7 +3541,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>67</v>
       </c>
@@ -3539,7 +3561,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>67</v>
       </c>
@@ -3559,7 +3581,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>67</v>
       </c>
@@ -3579,7 +3601,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>67</v>
       </c>
@@ -3599,7 +3621,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>67</v>
       </c>
@@ -3619,7 +3641,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>67</v>
       </c>
@@ -3639,7 +3661,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>67</v>
       </c>
@@ -3659,7 +3681,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>67</v>
       </c>
@@ -3679,7 +3701,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>67</v>
       </c>
@@ -3699,7 +3721,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>67</v>
       </c>
@@ -3767,7 +3789,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83D801B6-5B2D-4C63-87A9-B0F352D632BD}">
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="13.85546875" bestFit="1" customWidth="1"/>
@@ -3775,9 +3797,10 @@
     <col min="5" max="5" width="10.28515625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="76.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3799,8 +3822,11 @@
       <c r="G1" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H1" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -3815,7 +3841,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -3830,7 +3856,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -3852,7 +3878,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -3874,7 +3900,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -3896,7 +3922,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>44</v>
       </c>
@@ -3918,7 +3944,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>92</v>
       </c>
@@ -3940,7 +3966,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -3961,7 +3987,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>44</v>
       </c>
@@ -3986,7 +4012,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -4008,7 +4034,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>182</v>
       </c>
@@ -4030,7 +4056,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>151</v>
       </c>
@@ -4052,7 +4078,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>182</v>
       </c>
@@ -4074,7 +4100,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>196</v>
       </c>
@@ -4096,129 +4122,129 @@
         <v>200</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>151</v>
+      </c>
+      <c r="B16" t="s">
+        <v>67</v>
+      </c>
+      <c r="C16">
+        <f>beats!B56</f>
+        <v>64</v>
+      </c>
+      <c r="E16" t="s">
+        <v>67</v>
+      </c>
+      <c r="F16">
+        <f>beats!B56</f>
+        <v>64</v>
+      </c>
+      <c r="G16" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>182</v>
       </c>
-      <c r="B16" t="s">
-        <v>67</v>
-      </c>
-      <c r="C16">
+      <c r="B17" t="s">
+        <v>67</v>
+      </c>
+      <c r="C17">
         <f>beats!B57</f>
         <v>65</v>
       </c>
-      <c r="E16" t="s">
-        <v>67</v>
-      </c>
-      <c r="F16">
+      <c r="E17" t="s">
+        <v>67</v>
+      </c>
+      <c r="F17">
         <f>beats!B63</f>
         <v>71</v>
       </c>
-      <c r="G16" t="s">
+      <c r="G17" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>44</v>
       </c>
-      <c r="B17" t="s">
-        <v>67</v>
-      </c>
-      <c r="C17">
+      <c r="B18" t="s">
+        <v>67</v>
+      </c>
+      <c r="C18">
         <f>beats!B59</f>
         <v>67</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D18" t="s">
         <v>80</v>
       </c>
-      <c r="E17" t="s">
-        <v>67</v>
-      </c>
-      <c r="F17">
+      <c r="E18" t="s">
+        <v>67</v>
+      </c>
+      <c r="F18">
         <f>beats!B59</f>
         <v>67</v>
       </c>
-      <c r="G17" t="s">
+      <c r="G18" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
         <v>212</v>
       </c>
-      <c r="B18" t="s">
-        <v>67</v>
-      </c>
-      <c r="C18">
+      <c r="B19" t="s">
+        <v>67</v>
+      </c>
+      <c r="C19">
         <f>beats!B61</f>
         <v>69</v>
       </c>
-      <c r="E18" t="s">
-        <v>67</v>
-      </c>
-      <c r="F18">
+      <c r="E19" t="s">
+        <v>67</v>
+      </c>
+      <c r="F19">
         <f>beats!B61</f>
         <v>69</v>
       </c>
-      <c r="G18" t="s">
+      <c r="G19" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
         <v>182</v>
       </c>
-      <c r="B19" t="s">
-        <v>67</v>
-      </c>
-      <c r="C19">
+      <c r="B20" t="s">
+        <v>67</v>
+      </c>
+      <c r="C20">
         <f>beats!B63</f>
         <v>71</v>
       </c>
-      <c r="E19" t="s">
-        <v>67</v>
-      </c>
-      <c r="F19">
+      <c r="E20" t="s">
+        <v>67</v>
+      </c>
+      <c r="F20">
         <f>beats!B63</f>
         <v>71</v>
       </c>
-      <c r="G19" t="s">
+      <c r="G20" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>44</v>
       </c>
-      <c r="B20" t="s">
-        <v>67</v>
-      </c>
-      <c r="C20">
+      <c r="B21" t="s">
+        <v>67</v>
+      </c>
+      <c r="C21">
         <f>beats!B64</f>
         <v>72</v>
-      </c>
-      <c r="E20" t="s">
-        <v>67</v>
-      </c>
-      <c r="F20">
-        <f>beats!B66</f>
-        <v>74</v>
-      </c>
-      <c r="G20" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>224</v>
-      </c>
-      <c r="B21" t="s">
-        <v>67</v>
-      </c>
-      <c r="C21">
-        <f>beats!B65</f>
-        <v>73</v>
       </c>
       <c r="E21" t="s">
         <v>67</v>
@@ -4228,63 +4254,63 @@
         <v>74</v>
       </c>
       <c r="G21" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>224</v>
+      </c>
+      <c r="B22" t="s">
+        <v>67</v>
+      </c>
+      <c r="C22">
+        <f>beats!B65</f>
+        <v>73</v>
+      </c>
+      <c r="E22" t="s">
+        <v>67</v>
+      </c>
+      <c r="F22">
+        <f>beats!B66</f>
+        <v>74</v>
+      </c>
+      <c r="G22" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
         <v>182</v>
       </c>
-      <c r="B22" t="s">
-        <v>67</v>
-      </c>
-      <c r="C22">
+      <c r="B23" t="s">
+        <v>67</v>
+      </c>
+      <c r="C23">
         <f>beats!B68</f>
         <v>76</v>
       </c>
-      <c r="E22" t="s">
-        <v>67</v>
-      </c>
-      <c r="F22">
+      <c r="E23" t="s">
+        <v>67</v>
+      </c>
+      <c r="F23">
         <f>beats!B80</f>
         <v>88</v>
       </c>
-      <c r="G22" t="s">
+      <c r="G23" t="s">
         <v>291</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
         <v>44</v>
       </c>
-      <c r="B23" t="s">
-        <v>67</v>
-      </c>
-      <c r="C23">
+      <c r="B24" t="s">
+        <v>67</v>
+      </c>
+      <c r="C24">
         <f>beats!B71</f>
         <v>79</v>
-      </c>
-      <c r="E23" t="s">
-        <v>67</v>
-      </c>
-      <c r="F23">
-        <f>beats!B73</f>
-        <v>81</v>
-      </c>
-      <c r="G23" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>212</v>
-      </c>
-      <c r="B24" t="s">
-        <v>67</v>
-      </c>
-      <c r="C24">
-        <f>beats!B73</f>
-        <v>81</v>
       </c>
       <c r="E24" t="s">
         <v>67</v>
@@ -4294,37 +4320,34 @@
         <v>81</v>
       </c>
       <c r="G24" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>212</v>
+      </c>
+      <c r="B25" t="s">
+        <v>67</v>
+      </c>
+      <c r="C25">
+        <f>beats!B73</f>
+        <v>81</v>
+      </c>
+      <c r="E25" t="s">
+        <v>67</v>
+      </c>
+      <c r="F25">
+        <f>beats!B73</f>
+        <v>81</v>
+      </c>
+      <c r="G25" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
         <v>12</v>
-      </c>
-      <c r="B25" t="s">
-        <v>67</v>
-      </c>
-      <c r="C25">
-        <f>beats!B80</f>
-        <v>88</v>
-      </c>
-      <c r="D25" t="s">
-        <v>78</v>
-      </c>
-      <c r="E25" t="s">
-        <v>67</v>
-      </c>
-      <c r="F25">
-        <f>beats!B80</f>
-        <v>88</v>
-      </c>
-      <c r="G25" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>182</v>
       </c>
       <c r="B26" t="s">
         <v>67</v>
@@ -4344,7 +4367,38 @@
         <v>88</v>
       </c>
       <c r="G26" t="s">
+        <v>259</v>
+      </c>
+      <c r="H26" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>182</v>
+      </c>
+      <c r="B27" t="s">
+        <v>67</v>
+      </c>
+      <c r="C27">
+        <f>beats!B80</f>
+        <v>88</v>
+      </c>
+      <c r="D27" t="s">
+        <v>78</v>
+      </c>
+      <c r="E27" t="s">
+        <v>67</v>
+      </c>
+      <c r="F27">
+        <f>beats!B80</f>
+        <v>88</v>
+      </c>
+      <c r="G27" t="s">
         <v>250</v>
+      </c>
+      <c r="H27" t="s">
+        <v>296</v>
       </c>
     </row>
   </sheetData>
@@ -4355,7 +4409,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76C493BF-D343-46EF-AB39-E5F4461CCFFF}">
-  <dimension ref="A1:H45"/>
+  <dimension ref="A1:H47"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="15.85546875" bestFit="1" customWidth="1"/>
@@ -4802,6 +4856,9 @@
       <c r="A24" t="s">
         <v>12</v>
       </c>
+      <c r="B24" t="s">
+        <v>67</v>
+      </c>
       <c r="C24">
         <f>beats!B43</f>
         <v>51</v>
@@ -4817,6 +4874,9 @@
       <c r="A25" t="s">
         <v>151</v>
       </c>
+      <c r="B25" t="s">
+        <v>67</v>
+      </c>
       <c r="C25">
         <f>beats!B43</f>
         <v>51</v>
@@ -4832,6 +4892,9 @@
       <c r="A26" t="s">
         <v>182</v>
       </c>
+      <c r="B26" t="s">
+        <v>67</v>
+      </c>
       <c r="C26">
         <f>beats!B45</f>
         <v>53</v>
@@ -4850,6 +4913,9 @@
       <c r="A27" t="s">
         <v>92</v>
       </c>
+      <c r="B27" t="s">
+        <v>67</v>
+      </c>
       <c r="C27">
         <f>beats!B49</f>
         <v>57</v>
@@ -4865,6 +4931,9 @@
       <c r="A28" t="s">
         <v>196</v>
       </c>
+      <c r="B28" t="s">
+        <v>67</v>
+      </c>
       <c r="C28">
         <f>beats!B51</f>
         <v>59</v>
@@ -4880,6 +4949,9 @@
       <c r="A29" t="s">
         <v>182</v>
       </c>
+      <c r="B29" t="s">
+        <v>67</v>
+      </c>
       <c r="C29">
         <f>beats!B58</f>
         <v>66</v>
@@ -4895,6 +4967,9 @@
       <c r="A30" t="s">
         <v>212</v>
       </c>
+      <c r="B30" t="s">
+        <v>67</v>
+      </c>
       <c r="C30">
         <f>beats!B61</f>
         <v>69</v>
@@ -4910,6 +4985,9 @@
       <c r="A31" t="s">
         <v>12</v>
       </c>
+      <c r="B31" t="s">
+        <v>67</v>
+      </c>
       <c r="C31">
         <f>beats!B63</f>
         <v>71</v>
@@ -4925,6 +5003,9 @@
       <c r="A32" t="s">
         <v>182</v>
       </c>
+      <c r="B32" t="s">
+        <v>67</v>
+      </c>
       <c r="C32">
         <f>beats!B63</f>
         <v>71</v>
@@ -4940,6 +5021,9 @@
       <c r="A33" t="s">
         <v>224</v>
       </c>
+      <c r="B33" t="s">
+        <v>67</v>
+      </c>
       <c r="C33">
         <f>beats!B65</f>
         <v>73</v>
@@ -4948,190 +5032,263 @@
         <v>55</v>
       </c>
       <c r="E33" t="s">
-        <v>254</v>
+        <v>293</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>212</v>
+        <v>224</v>
+      </c>
+      <c r="B34" t="s">
+        <v>67</v>
       </c>
       <c r="C34">
-        <f>beats!B73</f>
-        <v>81</v>
+        <f>beats!B65</f>
+        <v>73</v>
       </c>
       <c r="D34" t="s">
         <v>55</v>
       </c>
       <c r="E34" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>44</v>
       </c>
+      <c r="B35" t="s">
+        <v>67</v>
+      </c>
       <c r="C35">
+        <f>beats!B65</f>
+        <v>73</v>
+      </c>
+      <c r="D35" t="s">
+        <v>55</v>
+      </c>
+      <c r="E35" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>212</v>
+      </c>
+      <c r="B36" t="s">
+        <v>67</v>
+      </c>
+      <c r="C36">
         <f>beats!B73</f>
         <v>81</v>
       </c>
-      <c r="D35" t="s">
+      <c r="D36" t="s">
         <v>55</v>
       </c>
-      <c r="E35" t="s">
+      <c r="E36" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>44</v>
+      </c>
+      <c r="B37" t="s">
+        <v>67</v>
+      </c>
+      <c r="C37">
+        <f>beats!B73</f>
+        <v>81</v>
+      </c>
+      <c r="D37" t="s">
+        <v>55</v>
+      </c>
+      <c r="E37" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
         <v>14</v>
       </c>
-      <c r="C36">
+      <c r="B38" t="s">
+        <v>67</v>
+      </c>
+      <c r="C38">
         <f>beats!B74</f>
         <v>82</v>
       </c>
-      <c r="D36" t="s">
+      <c r="D38" t="s">
         <v>55</v>
       </c>
-      <c r="E36" t="s">
+      <c r="E38" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
         <v>6</v>
       </c>
-      <c r="C37">
+      <c r="B39" t="s">
+        <v>67</v>
+      </c>
+      <c r="C39">
         <f>beats!B75</f>
         <v>83</v>
       </c>
-      <c r="D37" t="s">
+      <c r="D39" t="s">
         <v>55</v>
       </c>
-      <c r="E37" t="s">
+      <c r="E39" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
         <v>10</v>
       </c>
-      <c r="C38">
+      <c r="B40" t="s">
+        <v>67</v>
+      </c>
+      <c r="C40">
         <f>beats!B75</f>
         <v>83</v>
       </c>
-      <c r="D38" t="s">
-        <v>55</v>
-      </c>
-      <c r="E38" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>14</v>
-      </c>
-      <c r="C39">
-        <f>beats!B76</f>
-        <v>84</v>
-      </c>
-      <c r="D39" t="s">
-        <v>55</v>
-      </c>
-      <c r="E39" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>14</v>
-      </c>
-      <c r="C40">
-        <f>beats!B76</f>
-        <v>84</v>
-      </c>
       <c r="D40" t="s">
         <v>55</v>
       </c>
       <c r="E40" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>14</v>
       </c>
+      <c r="B41" t="s">
+        <v>67</v>
+      </c>
       <c r="C41">
+        <f>beats!B76</f>
+        <v>84</v>
+      </c>
+      <c r="D41" t="s">
+        <v>55</v>
+      </c>
+      <c r="E41" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>14</v>
+      </c>
+      <c r="B42" t="s">
+        <v>67</v>
+      </c>
+      <c r="C42">
+        <f>beats!B76</f>
+        <v>84</v>
+      </c>
+      <c r="D42" t="s">
+        <v>55</v>
+      </c>
+      <c r="E42" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>14</v>
+      </c>
+      <c r="B43" t="s">
+        <v>67</v>
+      </c>
+      <c r="C43">
         <f>beats!B77</f>
         <v>85</v>
       </c>
-      <c r="D41" t="s">
+      <c r="D43" t="s">
         <v>55</v>
       </c>
-      <c r="E41" t="s">
+      <c r="E43" t="s">
         <v>263</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
         <v>6</v>
       </c>
-      <c r="C42">
+      <c r="B44" t="s">
+        <v>67</v>
+      </c>
+      <c r="C44">
         <f>beats!B78</f>
         <v>86</v>
       </c>
-      <c r="D42" t="s">
+      <c r="D44" t="s">
         <v>55</v>
       </c>
-      <c r="E42" t="s">
+      <c r="E44" t="s">
         <v>264</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
         <v>10</v>
       </c>
-      <c r="C43">
+      <c r="B45" t="s">
+        <v>67</v>
+      </c>
+      <c r="C45">
         <f>beats!B78</f>
         <v>86</v>
       </c>
-      <c r="D43" t="s">
+      <c r="D45" t="s">
         <v>55</v>
       </c>
-      <c r="E43" t="s">
+      <c r="E45" t="s">
         <v>264</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
         <v>182</v>
       </c>
-      <c r="C44">
+      <c r="B46" t="s">
+        <v>67</v>
+      </c>
+      <c r="C46">
         <f>beats!B80</f>
         <v>88</v>
       </c>
-      <c r="D44" t="s">
+      <c r="D46" t="s">
         <v>55</v>
       </c>
-      <c r="E44" t="s">
+      <c r="E46" t="s">
         <v>265</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
         <v>12</v>
       </c>
-      <c r="C45">
+      <c r="B47" t="s">
+        <v>67</v>
+      </c>
+      <c r="C47">
         <f>beats!B80</f>
         <v>88</v>
       </c>
-      <c r="D45" t="s">
+      <c r="D47" t="s">
         <v>55</v>
       </c>
-      <c r="E45" t="s">
+      <c r="E47" t="s">
         <v>266</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
updated codex and routes
</commit_message>
<xml_diff>
--- a/TrailsTimeline.xlsx
+++ b/TrailsTimeline.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6da5a9201bc5826c/Documentos/trails_orbal_atlas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="765" documentId="13_ncr:1_{54315043-5A41-45C0-BA2E-F1BBE0C76030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A309053C-3586-48E4-AA7D-596D7AEC7E8E}"/>
+  <xr:revisionPtr revIDLastSave="799" documentId="13_ncr:1_{54315043-5A41-45C0-BA2E-F1BBE0C76030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D10308AF-B543-468A-9FC9-E7E745FB70F8}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{B6393BEF-99C0-4DAE-AD63-40B518CD1F0D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{B6393BEF-99C0-4DAE-AD63-40B518CD1F0D}"/>
   </bookViews>
   <sheets>
     <sheet name="characters" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="911" uniqueCount="297">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="926" uniqueCount="299">
   <si>
     <t>char_id</t>
   </si>
@@ -738,9 +738,6 @@
     <t>The party decide to go to Amberl Tower in search of their ship, only ot find it heavily guarded</t>
   </si>
   <si>
-    <t>Olivier interrupts while they are planning their assault, saying he will tag along regardless of the obstacles, and suggests sneaking into their ship, wich somehow works</t>
-  </si>
-  <si>
     <t>Finding a man named Lloyd who witnessed the Capua Sky Bandits alongside Valleria Lakeshore, and that they are coming back tonight</t>
   </si>
   <si>
@@ -759,9 +756,6 @@
     <t>Returning to Bose to report findings, received second recommendation letter</t>
   </si>
   <si>
-    <t>Also received a parcel intended for Cassius, with a black myserious orbment from someone named "K", and that he should take it to "R" for analysis</t>
-  </si>
-  <si>
     <t>ruan</t>
   </si>
   <si>
@@ -780,9 +774,6 @@
     <t>Part ways with Olivier and Scherazard who are going back to Rolent</t>
   </si>
   <si>
-    <t>After separating, Olivier is seen talking with someone about a mission on an orbment. Scherazard confronts him, and Olivier confesses he is involved with the Imperial Governmnet</t>
-  </si>
-  <si>
     <t>Chapter 2</t>
   </si>
   <si>
@@ -798,9 +789,6 @@
     <t>Going to Rolent with Scherazard</t>
   </si>
   <si>
-    <t>Defeated the Capua Sky Pirates, after which, their leader, and brother of Josette, states he has no memories of what happened after meeting THAT guy</t>
-  </si>
-  <si>
     <t>Taken away by the Intelligence Division</t>
   </si>
   <si>
@@ -825,9 +813,6 @@
     <t>Going to Rolent with Olivier</t>
   </si>
   <si>
-    <t>Received a parcel from Cassius with a letter stating they will find him if they keep climbing the bracer ranks, and that he cannot return until the end of the queen's birthday ceremony</t>
-  </si>
-  <si>
     <t>Left a letter for Estelle and Joshua explaining he cannot come back until the Queen's birthday cermony</t>
   </si>
   <si>
@@ -849,9 +834,6 @@
     <t>Setting out for Ruan</t>
   </si>
   <si>
-    <t>fc_ch3</t>
-  </si>
-  <si>
     <t>Stopping at the Krone Pass Checkpoint for the night</t>
   </si>
   <si>
@@ -873,9 +855,6 @@
     <t>letten</t>
   </si>
   <si>
-    <t>Air Lettern</t>
-  </si>
-  <si>
     <t>varenne</t>
   </si>
   <si>
@@ -934,6 +913,33 @@
   </si>
   <si>
     <t>air</t>
+  </si>
+  <si>
+    <t>Olivier interrupts while they are planning their assault</t>
+  </si>
+  <si>
+    <t>Olivier suggests sneaking into the ship, which somehow works</t>
+  </si>
+  <si>
+    <t>The Sky Bandit's leader, Josette's brother, says he has no memories of what happened after meeting THAT guy</t>
+  </si>
+  <si>
+    <t>Defeated the Capua Sky Pirates</t>
+  </si>
+  <si>
+    <t>After separating, Olivier is seen talking with someone about a mission on an orbment</t>
+  </si>
+  <si>
+    <t>Scherazard confronts Olivier, and Olivier confesses he is involved with the Imperial Governmnet</t>
+  </si>
+  <si>
+    <t>Also received a parcel intended for Cassius, with a black myserious orbment from someone named "K", and that he should take it to "R"</t>
+  </si>
+  <si>
+    <t>Received a parcel from Cassius urging them to keep climbing the ranks, and he cannot return until the queen's birthday ceremony</t>
+  </si>
+  <si>
+    <t>Air Letten</t>
   </si>
 </sst>
 </file>
@@ -1504,10 +1510,10 @@
         <v>67</v>
       </c>
       <c r="F8" t="s">
-        <v>285</v>
+        <v>278</v>
       </c>
       <c r="G8" t="s">
-        <v>283</v>
+        <v>276</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -1527,10 +1533,10 @@
         <v>67</v>
       </c>
       <c r="F9" t="s">
-        <v>286</v>
+        <v>279</v>
       </c>
       <c r="G9" t="s">
-        <v>287</v>
+        <v>280</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -1550,10 +1556,10 @@
         <v>67</v>
       </c>
       <c r="F10" t="s">
-        <v>288</v>
+        <v>281</v>
       </c>
       <c r="G10" t="s">
-        <v>284</v>
+        <v>277</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -1573,10 +1579,10 @@
         <v>67</v>
       </c>
       <c r="F11" t="s">
-        <v>289</v>
+        <v>282</v>
       </c>
       <c r="G11" t="s">
-        <v>290</v>
+        <v>283</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -1596,10 +1602,10 @@
         <v>67</v>
       </c>
       <c r="F12" t="s">
-        <v>282</v>
+        <v>275</v>
       </c>
       <c r="G12" t="s">
-        <v>281</v>
+        <v>274</v>
       </c>
     </row>
   </sheetData>
@@ -1958,10 +1964,10 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B18" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="C18" t="s">
         <v>23</v>
@@ -1972,13 +1978,13 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="B19" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="C19" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="D19" t="s">
         <v>24</v>
@@ -1992,13 +1998,13 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>270</v>
+        <v>264</v>
       </c>
       <c r="B20" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
       <c r="C20" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="D20" t="s">
         <v>40</v>
@@ -2012,13 +2018,13 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>272</v>
+        <v>266</v>
       </c>
       <c r="B21" t="s">
         <v>46</v>
       </c>
       <c r="C21" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="D21" t="s">
         <v>40</v>
@@ -2032,13 +2038,13 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>273</v>
+        <v>267</v>
       </c>
       <c r="B22" t="s">
-        <v>274</v>
+        <v>268</v>
       </c>
       <c r="C22" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="D22" t="s">
         <v>40</v>
@@ -2052,13 +2058,13 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>275</v>
+        <v>269</v>
       </c>
       <c r="B23" t="s">
-        <v>276</v>
+        <v>298</v>
       </c>
       <c r="C23" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="D23" t="s">
         <v>40</v>
@@ -2075,13 +2081,13 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
       <c r="B24" t="s">
-        <v>278</v>
+        <v>271</v>
       </c>
       <c r="C24" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="D24" t="s">
         <v>40</v>
@@ -2098,13 +2104,13 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>279</v>
+        <v>272</v>
       </c>
       <c r="B25" t="s">
-        <v>280</v>
+        <v>273</v>
       </c>
       <c r="C25" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="D25" t="s">
         <v>40</v>
@@ -2126,10 +2132,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{94EA2C8E-D265-418D-8065-F972E277CAB9}">
-  <dimension ref="A1:G82"/>
+  <dimension ref="A1:G85"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="162.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="144.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11.85546875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11.7109375" bestFit="1" customWidth="1"/>
@@ -2155,7 +2161,7 @@
         <v>32</v>
       </c>
       <c r="G1" t="s">
-        <v>295</v>
+        <v>288</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -3369,7 +3375,7 @@
         <v>68</v>
       </c>
       <c r="D62" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E62" t="s">
         <v>80</v>
@@ -3489,7 +3495,7 @@
         <v>68</v>
       </c>
       <c r="D68" t="s">
-        <v>231</v>
+        <v>290</v>
       </c>
       <c r="E68" t="s">
         <v>167</v>
@@ -3509,16 +3515,13 @@
         <v>68</v>
       </c>
       <c r="D69" t="s">
-        <v>248</v>
+        <v>291</v>
       </c>
       <c r="E69" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="F69" t="s">
         <v>69</v>
-      </c>
-      <c r="G69" t="s">
-        <v>296</v>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.25">
@@ -3532,7 +3535,7 @@
         <v>68</v>
       </c>
       <c r="D70" t="s">
-        <v>233</v>
+        <v>245</v>
       </c>
       <c r="E70" t="s">
         <v>163</v>
@@ -3540,6 +3543,9 @@
       <c r="F70" t="s">
         <v>69</v>
       </c>
+      <c r="G70" t="s">
+        <v>289</v>
+      </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
@@ -3552,7 +3558,7 @@
         <v>68</v>
       </c>
       <c r="D71" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="E71" t="s">
         <v>163</v>
@@ -3572,7 +3578,7 @@
         <v>68</v>
       </c>
       <c r="D72" t="s">
-        <v>251</v>
+        <v>233</v>
       </c>
       <c r="E72" t="s">
         <v>163</v>
@@ -3592,7 +3598,7 @@
         <v>68</v>
       </c>
       <c r="D73" t="s">
-        <v>236</v>
+        <v>293</v>
       </c>
       <c r="E73" t="s">
         <v>163</v>
@@ -3612,7 +3618,7 @@
         <v>68</v>
       </c>
       <c r="D74" t="s">
-        <v>235</v>
+        <v>292</v>
       </c>
       <c r="E74" t="s">
         <v>163</v>
@@ -3632,10 +3638,10 @@
         <v>68</v>
       </c>
       <c r="D75" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="E75" t="s">
-        <v>80</v>
+        <v>163</v>
       </c>
       <c r="F75" t="s">
         <v>69</v>
@@ -3652,10 +3658,10 @@
         <v>68</v>
       </c>
       <c r="D76" t="s">
-        <v>260</v>
+        <v>234</v>
       </c>
       <c r="E76" t="s">
-        <v>80</v>
+        <v>163</v>
       </c>
       <c r="F76" t="s">
         <v>69</v>
@@ -3672,7 +3678,7 @@
         <v>68</v>
       </c>
       <c r="D77" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="E77" t="s">
         <v>80</v>
@@ -3692,7 +3698,7 @@
         <v>68</v>
       </c>
       <c r="D78" t="s">
-        <v>243</v>
+        <v>297</v>
       </c>
       <c r="E78" t="s">
         <v>80</v>
@@ -3712,7 +3718,7 @@
         <v>68</v>
       </c>
       <c r="D79" t="s">
-        <v>244</v>
+        <v>296</v>
       </c>
       <c r="E79" t="s">
         <v>80</v>
@@ -3732,7 +3738,7 @@
         <v>68</v>
       </c>
       <c r="D80" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="E80" t="s">
         <v>80</v>
@@ -3743,16 +3749,16 @@
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>221</v>
+        <v>67</v>
       </c>
       <c r="B81">
         <v>89</v>
       </c>
       <c r="C81" t="s">
-        <v>246</v>
+        <v>68</v>
       </c>
       <c r="D81" t="s">
-        <v>267</v>
+        <v>242</v>
       </c>
       <c r="E81" t="s">
         <v>80</v>
@@ -3763,21 +3769,81 @@
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>268</v>
+        <v>67</v>
       </c>
       <c r="B82">
         <v>90</v>
       </c>
       <c r="C82" t="s">
-        <v>246</v>
+        <v>68</v>
       </c>
       <c r="D82" t="s">
-        <v>269</v>
+        <v>294</v>
       </c>
       <c r="E82" t="s">
+        <v>80</v>
+      </c>
+      <c r="F82" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>67</v>
+      </c>
+      <c r="B83">
+        <v>91</v>
+      </c>
+      <c r="C83" t="s">
+        <v>68</v>
+      </c>
+      <c r="D83" t="s">
+        <v>295</v>
+      </c>
+      <c r="E83" t="s">
+        <v>80</v>
+      </c>
+      <c r="F83" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>221</v>
+      </c>
+      <c r="B84">
+        <v>92</v>
+      </c>
+      <c r="C84" t="s">
+        <v>243</v>
+      </c>
+      <c r="D84" t="s">
+        <v>262</v>
+      </c>
+      <c r="E84" t="s">
+        <v>80</v>
+      </c>
+      <c r="F84" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>221</v>
+      </c>
+      <c r="B85">
+        <v>93</v>
+      </c>
+      <c r="C85" t="s">
+        <v>243</v>
+      </c>
+      <c r="D85" t="s">
+        <v>263</v>
+      </c>
+      <c r="E85" t="s">
         <v>171</v>
       </c>
-      <c r="F82" t="s">
+      <c r="F85" t="s">
         <v>69</v>
       </c>
     </row>
@@ -3823,7 +3889,7 @@
         <v>61</v>
       </c>
       <c r="H1" t="s">
-        <v>295</v>
+        <v>288</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -4027,8 +4093,8 @@
         <v>67</v>
       </c>
       <c r="F11">
-        <f>beats!B80</f>
-        <v>88</v>
+        <f>beats!B82</f>
+        <v>90</v>
       </c>
       <c r="G11" t="s">
         <v>149</v>
@@ -4137,11 +4203,11 @@
         <v>67</v>
       </c>
       <c r="F16">
-        <f>beats!B56</f>
-        <v>64</v>
+        <f>beats!B57</f>
+        <v>65</v>
       </c>
       <c r="G16" t="s">
-        <v>292</v>
+        <v>285</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
@@ -4254,7 +4320,7 @@
         <v>74</v>
       </c>
       <c r="G21" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
@@ -4276,7 +4342,7 @@
         <v>74</v>
       </c>
       <c r="G22" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
@@ -4294,11 +4360,11 @@
         <v>67</v>
       </c>
       <c r="F23">
-        <f>beats!B80</f>
-        <v>88</v>
+        <f>beats!B82</f>
+        <v>90</v>
       </c>
       <c r="G23" t="s">
-        <v>291</v>
+        <v>284</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
@@ -4309,18 +4375,18 @@
         <v>67</v>
       </c>
       <c r="C24">
-        <f>beats!B71</f>
-        <v>79</v>
+        <f>beats!B72</f>
+        <v>80</v>
       </c>
       <c r="E24" t="s">
         <v>67</v>
       </c>
       <c r="F24">
-        <f>beats!B73</f>
-        <v>81</v>
+        <f>beats!B75</f>
+        <v>83</v>
       </c>
       <c r="G24" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
@@ -4331,18 +4397,18 @@
         <v>67</v>
       </c>
       <c r="C25">
-        <f>beats!B73</f>
-        <v>81</v>
+        <f>beats!B75</f>
+        <v>83</v>
       </c>
       <c r="E25" t="s">
         <v>67</v>
       </c>
       <c r="F25">
-        <f>beats!B73</f>
-        <v>81</v>
+        <f>beats!B75</f>
+        <v>83</v>
       </c>
       <c r="G25" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
@@ -4353,8 +4419,8 @@
         <v>67</v>
       </c>
       <c r="C26">
-        <f>beats!B80</f>
-        <v>88</v>
+        <f>beats!B82</f>
+        <v>90</v>
       </c>
       <c r="D26" t="s">
         <v>78</v>
@@ -4363,14 +4429,14 @@
         <v>67</v>
       </c>
       <c r="F26">
-        <f>beats!B80</f>
-        <v>88</v>
+        <f>beats!B83</f>
+        <v>91</v>
       </c>
       <c r="G26" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
       <c r="H26" t="s">
-        <v>296</v>
+        <v>289</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
@@ -4381,8 +4447,8 @@
         <v>67</v>
       </c>
       <c r="C27">
-        <f>beats!B80</f>
-        <v>88</v>
+        <f>beats!B82</f>
+        <v>90</v>
       </c>
       <c r="D27" t="s">
         <v>78</v>
@@ -4391,14 +4457,14 @@
         <v>67</v>
       </c>
       <c r="F27">
-        <f>beats!B80</f>
-        <v>88</v>
+        <f>beats!B83</f>
+        <v>91</v>
       </c>
       <c r="G27" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="H27" t="s">
-        <v>296</v>
+        <v>289</v>
       </c>
     </row>
   </sheetData>
@@ -5032,7 +5098,7 @@
         <v>55</v>
       </c>
       <c r="E33" t="s">
-        <v>293</v>
+        <v>286</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
@@ -5050,7 +5116,7 @@
         <v>55</v>
       </c>
       <c r="E34" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
@@ -5068,7 +5134,7 @@
         <v>55</v>
       </c>
       <c r="E35" t="s">
-        <v>294</v>
+        <v>287</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
@@ -5079,14 +5145,14 @@
         <v>67</v>
       </c>
       <c r="C36">
-        <f>beats!B73</f>
-        <v>81</v>
+        <f>beats!B75</f>
+        <v>83</v>
       </c>
       <c r="D36" t="s">
         <v>55</v>
       </c>
       <c r="E36" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
@@ -5097,14 +5163,14 @@
         <v>67</v>
       </c>
       <c r="C37">
-        <f>beats!B73</f>
-        <v>81</v>
+        <f>beats!B75</f>
+        <v>83</v>
       </c>
       <c r="D37" t="s">
         <v>55</v>
       </c>
       <c r="E37" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
@@ -5115,14 +5181,14 @@
         <v>67</v>
       </c>
       <c r="C38">
-        <f>beats!B74</f>
-        <v>82</v>
+        <f>beats!B76</f>
+        <v>84</v>
       </c>
       <c r="D38" t="s">
         <v>55</v>
       </c>
       <c r="E38" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
@@ -5133,14 +5199,14 @@
         <v>67</v>
       </c>
       <c r="C39">
-        <f>beats!B75</f>
-        <v>83</v>
+        <f>beats!B77</f>
+        <v>85</v>
       </c>
       <c r="D39" t="s">
         <v>55</v>
       </c>
       <c r="E39" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
@@ -5151,14 +5217,14 @@
         <v>67</v>
       </c>
       <c r="C40">
-        <f>beats!B75</f>
-        <v>83</v>
+        <f>beats!B77</f>
+        <v>85</v>
       </c>
       <c r="D40" t="s">
         <v>55</v>
       </c>
       <c r="E40" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
@@ -5169,14 +5235,14 @@
         <v>67</v>
       </c>
       <c r="C41">
-        <f>beats!B76</f>
-        <v>84</v>
+        <f>beats!B78</f>
+        <v>86</v>
       </c>
       <c r="D41" t="s">
         <v>55</v>
       </c>
       <c r="E41" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
@@ -5187,14 +5253,14 @@
         <v>67</v>
       </c>
       <c r="C42">
-        <f>beats!B76</f>
-        <v>84</v>
+        <f>beats!B78</f>
+        <v>86</v>
       </c>
       <c r="D42" t="s">
         <v>55</v>
       </c>
       <c r="E42" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
@@ -5205,14 +5271,14 @@
         <v>67</v>
       </c>
       <c r="C43">
-        <f>beats!B77</f>
-        <v>85</v>
+        <f>beats!B79</f>
+        <v>87</v>
       </c>
       <c r="D43" t="s">
         <v>55</v>
       </c>
       <c r="E43" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
@@ -5223,14 +5289,14 @@
         <v>67</v>
       </c>
       <c r="C44">
-        <f>beats!B78</f>
-        <v>86</v>
+        <f>beats!B80</f>
+        <v>88</v>
       </c>
       <c r="D44" t="s">
         <v>55</v>
       </c>
       <c r="E44" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
@@ -5241,14 +5307,14 @@
         <v>67</v>
       </c>
       <c r="C45">
-        <f>beats!B78</f>
-        <v>86</v>
+        <f>beats!B80</f>
+        <v>88</v>
       </c>
       <c r="D45" t="s">
         <v>55</v>
       </c>
       <c r="E45" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
@@ -5259,14 +5325,14 @@
         <v>67</v>
       </c>
       <c r="C46">
-        <f>beats!B80</f>
-        <v>88</v>
+        <f>beats!B82</f>
+        <v>90</v>
       </c>
       <c r="D46" t="s">
         <v>55</v>
       </c>
       <c r="E46" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
@@ -5277,14 +5343,14 @@
         <v>67</v>
       </c>
       <c r="C47">
-        <f>beats!B80</f>
-        <v>88</v>
+        <f>beats!B82</f>
+        <v>90</v>
       </c>
       <c r="D47" t="s">
         <v>55</v>
       </c>
       <c r="E47" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
     </row>
   </sheetData>

</xml_diff>